<commit_message>
Checkpoint: Series A sheet with formula-driven SAFE conversion and option pool expansion
</commit_message>
<xml_diff>
--- a/runs/resume/models/model.xlsx
+++ b/runs/resume/models/model.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{69A5EB88-CD2C-2C43-A1C7-5B8131726479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{69D6012A-AD98-E548-9F95-626803C86B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sidekick Cap Table" sheetId="19" r:id="rId1"/>
     <sheet name="SAFE Investments" sheetId="20" r:id="rId2"/>
+    <sheet name="Series A" sheetId="24" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="98">
   <si>
     <t>Total</t>
   </si>
@@ -193,13 +194,152 @@
   </si>
   <si>
     <t>Mark Lotke</t>
+  </si>
+  <si>
+    <t>Series A</t>
+  </si>
+  <si>
+    <t>Total Capitalization</t>
+  </si>
+  <si>
+    <t># of</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Preferred</t>
+  </si>
+  <si>
+    <t>Pool +</t>
+  </si>
+  <si>
+    <t>Total FD</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Shares</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Invested</t>
+  </si>
+  <si>
+    <t>Pre A</t>
+  </si>
+  <si>
+    <t>FD</t>
+  </si>
+  <si>
+    <t>Common Stock and Options:</t>
+  </si>
+  <si>
+    <t>Total Common</t>
+  </si>
+  <si>
+    <t>Preferred Rounds</t>
+  </si>
+  <si>
+    <t>1011 Ventures</t>
+  </si>
+  <si>
+    <t>Other Series A Investors</t>
+  </si>
+  <si>
+    <t>Totals</t>
+  </si>
+  <si>
+    <t>Price per Share</t>
+  </si>
+  <si>
+    <t>Pre-Money Valuation</t>
+  </si>
+  <si>
+    <t>Post-Money Valuation</t>
+  </si>
+  <si>
+    <t>Series A Assumptions:</t>
+  </si>
+  <si>
+    <t>Total Raised</t>
+  </si>
+  <si>
+    <t>1011 Ventures Investment</t>
+  </si>
+  <si>
+    <t>Accomplice Investment</t>
+  </si>
+  <si>
+    <t>SAFE Post-Money Valuation Cap</t>
+  </si>
+  <si>
+    <t>Common</t>
+  </si>
+  <si>
+    <t>Option</t>
+  </si>
+  <si>
+    <t>SIDEKICK (THINK MORE SECURITY) &amp; 1011/ACCOMPLICE SERIES A</t>
+  </si>
+  <si>
+    <t>Other Common Shareholders</t>
+  </si>
+  <si>
+    <t>ESOP Available</t>
+  </si>
+  <si>
+    <t>Accomplice (Affiliated Funds)</t>
+  </si>
+  <si>
+    <t>Other SAFE Investors</t>
+  </si>
+  <si>
+    <t>Other Series A Investment</t>
+  </si>
+  <si>
+    <t>Option Pool Target (% Post-Money)</t>
+  </si>
+  <si>
+    <t>Existing Unallocated Options</t>
+  </si>
+  <si>
+    <t>New Option Pool Shares</t>
+  </si>
+  <si>
+    <t>Pre-existing Capitalization</t>
+  </si>
+  <si>
+    <t>Total SAFE Invested</t>
+  </si>
+  <si>
+    <t>SAFE Price per Share</t>
+  </si>
+  <si>
+    <t>Total SAFE Conversion Shares</t>
+  </si>
+  <si>
+    <t>Total Post-Money FD Shares</t>
+  </si>
+  <si>
+    <t>Series A Price per Share</t>
+  </si>
+  <si>
+    <t>Total Series A Shares</t>
+  </si>
+  <si>
+    <t>Check (Investments = Total Raised)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0000"/>
+  </numFmts>
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -335,14 +475,28 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF008000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -525,6 +679,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -709,19 +869,33 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="18" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="18" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1128,38 +1302,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3" t="s">
+      <c r="A1" s="7"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4" t="s">
+      <c r="A2" s="8"/>
+      <c r="B2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="8" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1167,16 +1341,16 @@
       <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="2">
         <v>3600000</v>
       </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1">
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2">
         <v>3600000</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="3">
         <v>0.36959987630724139</v>
       </c>
     </row>
@@ -1184,16 +1358,16 @@
       <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <v>3600000</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1">
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2">
         <v>3600000</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="3">
         <v>0.36959987630724139</v>
       </c>
     </row>
@@ -1201,16 +1375,16 @@
       <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="2">
         <v>222187</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1">
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2">
         <v>222187</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="3">
         <v>2.28111910325214E-2</v>
       </c>
     </row>
@@ -1218,16 +1392,16 @@
       <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="2">
         <v>592500</v>
       </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1">
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2">
         <v>592500</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="3">
         <v>6.0829979642233481E-2</v>
       </c>
     </row>
@@ -1235,16 +1409,16 @@
       <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="2">
         <v>592500</v>
       </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1">
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2">
         <v>592500</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="3">
         <v>6.0829979642233481E-2</v>
       </c>
     </row>
@@ -1252,18 +1426,18 @@
       <c r="B8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="2">
         <v>13500</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>98900</v>
       </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1">
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2">
         <v>112400</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="3">
         <v>1.1539729471370537E-2</v>
       </c>
     </row>
@@ -1271,16 +1445,16 @@
       <c r="B9" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="2">
         <v>9000</v>
       </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1">
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2">
         <v>9000</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="3">
         <v>9.2399969076810353E-4</v>
       </c>
     </row>
@@ -1288,16 +1462,16 @@
       <c r="B10" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1">
+      <c r="C10" s="2"/>
+      <c r="D10" s="2">
         <v>95000</v>
       </c>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1">
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2">
         <v>95000</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="3">
         <v>9.7533300692188695E-3</v>
       </c>
     </row>
@@ -1305,16 +1479,16 @@
       <c r="B11" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1">
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2">
         <v>25000</v>
       </c>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1">
+      <c r="F11" s="2"/>
+      <c r="G11" s="2">
         <v>25000</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="3">
         <v>2.5666658076891765E-3</v>
       </c>
     </row>
@@ -1322,16 +1496,16 @@
       <c r="B12" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1">
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2">
         <v>41562</v>
       </c>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1">
+      <c r="F12" s="2"/>
+      <c r="G12" s="2">
         <v>41562</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="3">
         <v>4.2670305719671019E-3</v>
       </c>
     </row>
@@ -1339,16 +1513,16 @@
       <c r="B13" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1">
+      <c r="C13" s="2"/>
+      <c r="D13" s="2">
         <v>285000</v>
       </c>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1">
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2">
         <v>285000</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="3">
         <v>2.925999020765661E-2</v>
       </c>
     </row>
@@ -1356,16 +1530,16 @@
       <c r="B14" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1">
+      <c r="C14" s="2"/>
+      <c r="D14" s="2">
         <v>50000</v>
       </c>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1">
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2">
         <v>50000</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="3">
         <v>5.133331615378353E-3</v>
       </c>
     </row>
@@ -1373,16 +1547,16 @@
       <c r="B15" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1">
+      <c r="C15" s="2"/>
+      <c r="D15" s="2">
         <v>285000</v>
       </c>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1">
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2">
         <v>285000</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="3">
         <v>2.925999020765661E-2</v>
       </c>
     </row>
@@ -1390,16 +1564,16 @@
       <c r="B16" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1">
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2">
         <v>96186</v>
       </c>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1">
+      <c r="F16" s="2"/>
+      <c r="G16" s="2">
         <v>96186</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="3">
         <v>9.8750926951356455E-3</v>
       </c>
     </row>
@@ -1407,16 +1581,16 @@
       <c r="B17" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1">
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2">
         <v>48095</v>
       </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1">
+      <c r="F17" s="2"/>
+      <c r="G17" s="2">
         <v>48095</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="3">
         <v>4.9377516808324371E-3</v>
       </c>
     </row>
@@ -1424,16 +1598,16 @@
       <c r="B18" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1">
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2">
         <v>12395</v>
       </c>
-      <c r="G18" s="1">
+      <c r="G18" s="2">
         <v>12395</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="3">
         <v>1.2725529074522936E-3</v>
       </c>
     </row>
@@ -1441,16 +1615,16 @@
       <c r="B19" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1">
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2">
         <v>8333</v>
       </c>
-      <c r="G19" s="1">
+      <c r="G19" s="2">
         <v>8333</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="3">
         <v>8.5552104701895626E-4</v>
       </c>
     </row>
@@ -1458,40 +1632,40 @@
       <c r="B20" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1">
+      <c r="C20" s="2"/>
+      <c r="D20" s="2">
         <v>65105</v>
       </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1">
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2">
         <v>65105</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="3">
         <v>6.6841110963841528E-3</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5" t="s">
+      <c r="A21" s="9"/>
+      <c r="B21" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="10">
         <v>8629687</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="10">
         <v>879005</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="10">
         <v>210843</v>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="10">
         <v>20728</v>
       </c>
-      <c r="G21" s="6">
+      <c r="G21" s="10">
         <v>9740263</v>
       </c>
-      <c r="H21" s="7"/>
+      <c r="H21" s="11"/>
     </row>
     <row r="22" spans="1:8" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
@@ -1512,15 +1686,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4" t="s">
+      <c r="A1" s="8"/>
+      <c r="B1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="D1" s="8"/>
+      <c r="E1" s="8" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1528,7 +1702,7 @@
       <c r="B2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="2">
         <v>25000</v>
       </c>
       <c r="E2" t="s">
@@ -1539,7 +1713,7 @@
       <c r="B3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="2">
         <v>25000</v>
       </c>
     </row>
@@ -1547,7 +1721,7 @@
       <c r="B4" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <v>137170.75</v>
       </c>
     </row>
@@ -1555,7 +1729,7 @@
       <c r="B5" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="2">
         <v>3846829.25</v>
       </c>
     </row>
@@ -1563,7 +1737,7 @@
       <c r="B6" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="2">
         <v>16566</v>
       </c>
       <c r="E6" t="s">
@@ -1574,7 +1748,7 @@
       <c r="B7" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="2">
         <v>250000</v>
       </c>
     </row>
@@ -1582,7 +1756,7 @@
       <c r="B8" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="2">
         <v>100000</v>
       </c>
     </row>
@@ -1590,7 +1764,7 @@
       <c r="B9" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="2">
         <v>300000</v>
       </c>
       <c r="E9" t="s">
@@ -1601,7 +1775,7 @@
       <c r="B10" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="2">
         <v>37500</v>
       </c>
       <c r="E10" t="s">
@@ -1612,7 +1786,7 @@
       <c r="B11" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="2">
         <v>250000</v>
       </c>
     </row>
@@ -1620,7 +1794,7 @@
       <c r="B12" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="2">
         <v>100000</v>
       </c>
     </row>
@@ -1628,7 +1802,7 @@
       <c r="B13" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="2">
         <v>41164</v>
       </c>
       <c r="E13" t="s">
@@ -1639,7 +1813,7 @@
       <c r="B14" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="2">
         <v>2328778</v>
       </c>
       <c r="E14" t="s">
@@ -1650,7 +1824,7 @@
       <c r="B15" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="2">
         <v>1506000</v>
       </c>
       <c r="E15" t="s">
@@ -1661,7 +1835,7 @@
       <c r="B16" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="2">
         <v>50000</v>
       </c>
     </row>
@@ -1669,7 +1843,7 @@
       <c r="B17" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="2">
         <v>212500</v>
       </c>
       <c r="E17" t="s">
@@ -1680,7 +1854,7 @@
       <c r="B18" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" s="2">
         <v>25000</v>
       </c>
     </row>
@@ -1688,7 +1862,7 @@
       <c r="B19" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" s="2">
         <v>61746</v>
       </c>
       <c r="E19" t="s">
@@ -1699,7 +1873,7 @@
       <c r="B20" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="2">
         <v>100000</v>
       </c>
     </row>
@@ -1707,7 +1881,7 @@
       <c r="B21" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21" s="2">
         <v>100000</v>
       </c>
     </row>
@@ -1715,7 +1889,7 @@
       <c r="B22" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22" s="2">
         <v>61746</v>
       </c>
       <c r="E22" t="s">
@@ -1726,7 +1900,7 @@
       <c r="B23" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" s="2">
         <v>250000</v>
       </c>
       <c r="E23" t="s">
@@ -1734,18 +1908,894 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5" t="s">
+      <c r="A24" s="9"/>
+      <c r="B24" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="10">
         <v>9825000</v>
       </c>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
     </row>
     <row r="25" spans="1:5" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BDD7B37-73DF-F641-9F36-44DBA8C4C9E2}">
+  <dimension ref="A1:M53"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="3.83203125" customWidth="1"/>
+    <col min="2" max="2" width="51.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.83203125" customWidth="1"/>
+    <col min="7" max="8" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.83203125" customWidth="1"/>
+    <col min="10" max="10" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.83203125" customWidth="1"/>
+    <col min="12" max="12" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B1" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="M3" s="7"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" s="12"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="M5" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B6" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="19">
+        <f>'Sidekick Cap Table'!G3</f>
+        <v>3600000</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="L7" s="2">
+        <f>C7</f>
+        <v>3600000</v>
+      </c>
+      <c r="M7" s="3">
+        <f>L7/$C$49</f>
+        <v>0.2019135244706487</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="19">
+        <f>'Sidekick Cap Table'!G4</f>
+        <v>3600000</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="L8" s="2">
+        <f>C8</f>
+        <v>3600000</v>
+      </c>
+      <c r="M8" s="3">
+        <f>L8/$C$49</f>
+        <v>0.2019135244706487</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="19">
+        <f>'Sidekick Cap Table'!G6</f>
+        <v>592500</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="L9" s="2">
+        <f>C9</f>
+        <v>592500</v>
+      </c>
+      <c r="M9" s="3">
+        <f>L9/$C$49</f>
+        <v>3.3231600902460932E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="19">
+        <f>'Sidekick Cap Table'!G7</f>
+        <v>592500</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="L10" s="2">
+        <f>C10</f>
+        <v>592500</v>
+      </c>
+      <c r="M10" s="3">
+        <f>L10/$C$49</f>
+        <v>3.3231600902460932E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="19">
+        <f>'Sidekick Cap Table'!G5</f>
+        <v>222187</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="L11" s="2">
+        <f>C11</f>
+        <v>222187</v>
+      </c>
+      <c r="M11" s="3">
+        <f>L11/$C$49</f>
+        <v>1.2461822294877785E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="19">
+        <f>'Sidekick Cap Table'!G13</f>
+        <v>285000</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="L12" s="2">
+        <f>C12</f>
+        <v>285000</v>
+      </c>
+      <c r="M12" s="3">
+        <f>L12/$C$49</f>
+        <v>1.598482068725969E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="19">
+        <f>'Sidekick Cap Table'!G15</f>
+        <v>285000</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="L13" s="2">
+        <f>C13</f>
+        <v>285000</v>
+      </c>
+      <c r="M13" s="3">
+        <f>L13/$C$49</f>
+        <v>1.598482068725969E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="19">
+        <f>'Sidekick Cap Table'!G8</f>
+        <v>112400</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="L14" s="2">
+        <f>C14</f>
+        <v>112400</v>
+      </c>
+      <c r="M14" s="3">
+        <f>L14/$C$49</f>
+        <v>6.3041889306946989E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="19">
+        <f>'Sidekick Cap Table'!G9+'Sidekick Cap Table'!G10+'Sidekick Cap Table'!G11+'Sidekick Cap Table'!G12+'Sidekick Cap Table'!G14+'Sidekick Cap Table'!G16+'Sidekick Cap Table'!G17+'Sidekick Cap Table'!G18+'Sidekick Cap Table'!G19</f>
+        <v>385571</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="L15" s="2">
+        <f>C15</f>
+        <v>385571</v>
+      </c>
+      <c r="M15" s="3">
+        <f>L15/$C$49</f>
+        <v>2.1625555428797915E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="19">
+        <f>'Sidekick Cap Table'!G20</f>
+        <v>65105</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="J16" s="2">
+        <f>$C$52</f>
+        <v>1717836.4891538464</v>
+      </c>
+      <c r="L16" s="2">
+        <f>C16+J16</f>
+        <v>1782941.4891538464</v>
+      </c>
+      <c r="M16" s="3">
+        <f>L16/$C$49</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B17" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" s="4">
+        <f>SUM(C7:C16)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="4">
+        <f>SUM(J7:J16)</f>
+        <v>1717836.4891538464</v>
+      </c>
+      <c r="K17" s="1"/>
+      <c r="L17" s="4">
+        <f>SUM(L7:L16)</f>
+        <v>11458099.489153847</v>
+      </c>
+      <c r="M17" s="5">
+        <f>L17/$C$49</f>
+        <v>0.6426514587751091</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="3"/>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="3"/>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="19">
+        <f>'SAFE Investments'!C4+'SAFE Investments'!C5+'SAFE Investments'!C6+'SAFE Investments'!C13+'SAFE Investments'!C14+'SAFE Investments'!C15+'SAFE Investments'!C19+'SAFE Investments'!C22</f>
+        <v>8000000</v>
+      </c>
+      <c r="E20" s="2">
+        <f>D20/$C$47</f>
+        <v>1558442.08</v>
+      </c>
+      <c r="G20" s="2">
+        <f>$C$39</f>
+        <v>5000000</v>
+      </c>
+      <c r="H20" s="2">
+        <f>G20/$C$50</f>
+        <v>1114338.430721154</v>
+      </c>
+      <c r="J20" s="2"/>
+      <c r="L20" s="2">
+        <f>E20+H20</f>
+        <v>2672780.510721154</v>
+      </c>
+      <c r="M20" s="3">
+        <f>L20/$C$49</f>
+        <v>0.14990848140449131</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B21" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="19">
+        <f>'SAFE Investments'!C7</f>
+        <v>250000</v>
+      </c>
+      <c r="E21" s="2">
+        <f>D21/$C$47</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="L21" s="2">
+        <f>E21</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="M21" s="3">
+        <f>L21/$C$49</f>
+        <v>2.7315150438903531E-3</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="19">
+        <f>'SAFE Investments'!C9</f>
+        <v>300000</v>
+      </c>
+      <c r="E22" s="2">
+        <f>D22/$C$47</f>
+        <v>58441.578000000001</v>
+      </c>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="L22" s="2">
+        <f>E22</f>
+        <v>58441.578000000001</v>
+      </c>
+      <c r="M22" s="3">
+        <f>L22/$C$49</f>
+        <v>3.2778180526684235E-3</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" s="19">
+        <f>'SAFE Investments'!C11</f>
+        <v>250000</v>
+      </c>
+      <c r="E23" s="2">
+        <f>D23/$C$47</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="L23" s="2">
+        <f>E23</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="M23" s="3">
+        <f>L23/$C$49</f>
+        <v>2.7315150438903531E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="19">
+        <f>'SAFE Investments'!C17</f>
+        <v>212500</v>
+      </c>
+      <c r="E24" s="2">
+        <f>D24/$C$47</f>
+        <v>41396.117749999998</v>
+      </c>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="L24" s="2">
+        <f>E24</f>
+        <v>41396.117749999998</v>
+      </c>
+      <c r="M24" s="3">
+        <f>L24/$C$49</f>
+        <v>2.3217877873068001E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B25" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="19">
+        <f>'SAFE Investments'!C23</f>
+        <v>250000</v>
+      </c>
+      <c r="E25" s="2">
+        <f>D25/$C$47</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="L25" s="2">
+        <f>E25</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="M25" s="3">
+        <f>L25/$C$49</f>
+        <v>2.7315150438903531E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>85</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="19">
+        <f>'SAFE Investments'!C2+'SAFE Investments'!C3+'SAFE Investments'!C8+'SAFE Investments'!C10+'SAFE Investments'!C12+'SAFE Investments'!C16+'SAFE Investments'!C18+'SAFE Investments'!C20+'SAFE Investments'!C21</f>
+        <v>562500</v>
+      </c>
+      <c r="E26" s="2">
+        <f>D26/$C$47</f>
+        <v>109577.95875000001</v>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="L26" s="2">
+        <f>E26</f>
+        <v>109577.95875000001</v>
+      </c>
+      <c r="M26" s="3">
+        <f>L26/$C$49</f>
+        <v>6.1459088487532945E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B27" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="G27" s="2">
+        <f>$C$38</f>
+        <v>12000000</v>
+      </c>
+      <c r="H27" s="2">
+        <f>G27/$C$50</f>
+        <v>2674412.2337307697</v>
+      </c>
+      <c r="J27" s="2"/>
+      <c r="L27" s="2">
+        <f>H27</f>
+        <v>2674412.2337307697</v>
+      </c>
+      <c r="M27" s="3">
+        <f>L27/$C$49</f>
+        <v>0.15000000000000002</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B28" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="G28" s="2">
+        <f>$C$40</f>
+        <v>3000000</v>
+      </c>
+      <c r="H28" s="2">
+        <f>G28/$C$50</f>
+        <v>668603.05843269243</v>
+      </c>
+      <c r="J28" s="2"/>
+      <c r="L28" s="2">
+        <f>H28</f>
+        <v>668603.05843269243</v>
+      </c>
+      <c r="M28" s="3">
+        <f>L28/$C$49</f>
+        <v>3.7500000000000006E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="J29" s="2"/>
+      <c r="L29" s="2"/>
+      <c r="M29" s="3"/>
+    </row>
+    <row r="30" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30" s="16">
+        <f>SUM(C7:C16)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D30" s="16">
+        <f>SUM(D20:D26)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E30" s="16">
+        <f>SUM(E20:E26)</f>
+        <v>1913961.6794999999</v>
+      </c>
+      <c r="F30" s="13"/>
+      <c r="G30" s="16">
+        <f>SUM(G20:G28)</f>
+        <v>20000000</v>
+      </c>
+      <c r="H30" s="16">
+        <f>SUM(H20:H28)</f>
+        <v>4457353.7228846159</v>
+      </c>
+      <c r="I30" s="13"/>
+      <c r="J30" s="16">
+        <f>J16</f>
+        <v>1717836.4891538464</v>
+      </c>
+      <c r="K30" s="13"/>
+      <c r="L30" s="16">
+        <f>C30+E30+H30+J30</f>
+        <v>17829414.891538464</v>
+      </c>
+      <c r="M30" s="17">
+        <f>L30/$C$49</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E32" s="18">
+        <f>$C$47</f>
+        <v>5.1333316153783528</v>
+      </c>
+      <c r="H32" s="18">
+        <f>$C$50</f>
+        <v>4.48696721045886</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E33" s="2">
+        <f>$C$42</f>
+        <v>50000000</v>
+      </c>
+      <c r="H33" s="2">
+        <f>$C$36</f>
+        <v>60000000</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B34" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E34" s="2">
+        <f>$C$42</f>
+        <v>50000000</v>
+      </c>
+      <c r="H34" s="2">
+        <f>$C$41</f>
+        <v>80000000</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B35" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B36" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="14">
+        <v>60000000</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B37" t="s">
+        <v>75</v>
+      </c>
+      <c r="C37" s="14">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B38" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" s="14">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>77</v>
+      </c>
+      <c r="C39" s="14">
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40" s="14">
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B41" t="s">
+        <v>73</v>
+      </c>
+      <c r="C41" s="2">
+        <f>C36+C37</f>
+        <v>80000000</v>
+      </c>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>78</v>
+      </c>
+      <c r="C42" s="14">
+        <v>50000000</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
+        <v>87</v>
+      </c>
+      <c r="C43" s="15">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
+        <v>90</v>
+      </c>
+      <c r="C44" s="19">
+        <f>'Sidekick Cap Table'!G21</f>
+        <v>9740263</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
+        <v>91</v>
+      </c>
+      <c r="C45" s="19">
+        <f>'SAFE Investments'!C24</f>
+        <v>9825000</v>
+      </c>
+    </row>
+    <row r="46" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B46" t="s">
+        <v>88</v>
+      </c>
+      <c r="C46" s="19">
+        <f>'Sidekick Cap Table'!G20</f>
+        <v>65105</v>
+      </c>
+    </row>
+    <row r="47" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B47" t="s">
+        <v>92</v>
+      </c>
+      <c r="C47" s="18">
+        <f>C42/C44</f>
+        <v>5.1333316153783528</v>
+      </c>
+    </row>
+    <row r="48" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B48" t="s">
+        <v>93</v>
+      </c>
+      <c r="C48" s="2">
+        <f>C45/C47</f>
+        <v>1913961.6794999999</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B49" t="s">
+        <v>94</v>
+      </c>
+      <c r="C49" s="2">
+        <f>(C44+C48-C46)/(1-C43-C37/C41)</f>
+        <v>17829414.891538464</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B50" t="s">
+        <v>95</v>
+      </c>
+      <c r="C50" s="18">
+        <f>C41/C49</f>
+        <v>4.48696721045886</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B51" t="s">
+        <v>96</v>
+      </c>
+      <c r="C51" s="2">
+        <f>C37/C50</f>
+        <v>4457353.7228846159</v>
+      </c>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B52" t="s">
+        <v>89</v>
+      </c>
+      <c r="C52" s="2">
+        <f>C43*C49-C46</f>
+        <v>1717836.4891538464</v>
+      </c>
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B53" t="s">
+        <v>97</v>
+      </c>
+      <c r="C53" s="2">
+        <f>C38+C39+C40-C37</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Checkpoint: Series B sheet with pro rata allocation and option pool gross top-up
</commit_message>
<xml_diff>
--- a/runs/resume/models/model.xlsx
+++ b/runs/resume/models/model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{69D6012A-AD98-E548-9F95-626803C86B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2B8674A8-8D31-A842-80F7-DC0C9C95F142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sidekick Cap Table" sheetId="19" r:id="rId1"/>
     <sheet name="SAFE Investments" sheetId="20" r:id="rId2"/>
     <sheet name="Series A" sheetId="24" r:id="rId3"/>
+    <sheet name="Series B" sheetId="25" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="116">
   <si>
     <t>Total</t>
   </si>
@@ -274,6 +275,15 @@
     <t>SAFE Post-Money Valuation Cap</t>
   </si>
   <si>
+    <t>Series B</t>
+  </si>
+  <si>
+    <t>Pre B</t>
+  </si>
+  <si>
+    <t>Series B Assumptions:</t>
+  </si>
+  <si>
     <t>Common</t>
   </si>
   <si>
@@ -329,6 +339,51 @@
   </si>
   <si>
     <t>Check (Investments = Total Raised)</t>
+  </si>
+  <si>
+    <t>Other Series B Investment</t>
+  </si>
+  <si>
+    <t>Remaining for Pro Rata</t>
+  </si>
+  <si>
+    <t>Option Pool Gross Top-Up (%)</t>
+  </si>
+  <si>
+    <t>Post-A Total FD Shares</t>
+  </si>
+  <si>
+    <t>Post-A ESOP Available</t>
+  </si>
+  <si>
+    <t>Series B Price per Share</t>
+  </si>
+  <si>
+    <t>Total Series B Shares</t>
+  </si>
+  <si>
+    <t>Post-B FD (before option top-up)</t>
+  </si>
+  <si>
+    <t>Post-B Total FD Shares</t>
+  </si>
+  <si>
+    <t>New Option Pool Shares (Gross Top-Up)</t>
+  </si>
+  <si>
+    <t>1011 Pro Rata B Investment</t>
+  </si>
+  <si>
+    <t>Accomplice Pro Rata B Investment</t>
+  </si>
+  <si>
+    <t>Other A Investors Pro Rata B Investment</t>
+  </si>
+  <si>
+    <t>SIDEKICK (THINK MORE SECURITY) &amp; 1011/ACCOMPLICE SERIES B</t>
+  </si>
+  <si>
+    <t>Other Series B Investors</t>
   </si>
 </sst>
 </file>
@@ -869,7 +924,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -896,6 +951,8 @@
     <xf numFmtId="10" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1945,14 +2002,14 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B1" s="6" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="7" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>26</v>
@@ -1965,7 +2022,7 @@
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
       <c r="J3" s="7" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K3" s="7"/>
       <c r="L3" s="7" t="s">
@@ -2218,7 +2275,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C15" s="19">
         <f>'Sidekick Cap Table'!G9+'Sidekick Cap Table'!G10+'Sidekick Cap Table'!G11+'Sidekick Cap Table'!G12+'Sidekick Cap Table'!G14+'Sidekick Cap Table'!G16+'Sidekick Cap Table'!G17+'Sidekick Cap Table'!G18+'Sidekick Cap Table'!G19</f>
@@ -2240,7 +2297,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C16" s="19">
         <f>'Sidekick Cap Table'!G20</f>
@@ -2316,7 +2373,7 @@
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="19">
@@ -2472,7 +2529,7 @@
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="19">
@@ -2674,7 +2731,7 @@
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C40" s="14">
         <v>3000000</v>
@@ -2699,7 +2756,7 @@
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C43" s="15">
         <v>0.1</v>
@@ -2707,7 +2764,7 @@
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C44" s="19">
         <f>'Sidekick Cap Table'!G21</f>
@@ -2716,7 +2773,7 @@
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C45" s="19">
         <f>'SAFE Investments'!C24</f>
@@ -2725,7 +2782,7 @@
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C46" s="19">
         <f>'Sidekick Cap Table'!G20</f>
@@ -2734,7 +2791,7 @@
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C47" s="18">
         <f>C42/C44</f>
@@ -2743,7 +2800,7 @@
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C48" s="2">
         <f>C45/C47</f>
@@ -2752,7 +2809,7 @@
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C49" s="2">
         <f>(C44+C48-C46)/(1-C43-C37/C41)</f>
@@ -2761,7 +2818,7 @@
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C50" s="18">
         <f>C41/C49</f>
@@ -2770,7 +2827,7 @@
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C51" s="2">
         <f>C37/C50</f>
@@ -2779,7 +2836,7 @@
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C52" s="2">
         <f>C43*C49-C46</f>
@@ -2788,11 +2845,1040 @@
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C53" s="2">
         <f>C38+C39+C40-C37</f>
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AF22BCC-A6D7-6749-9B46-9E072129FD10}">
+  <dimension ref="A1:R51"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="3.83203125" customWidth="1"/>
+    <col min="2" max="2" width="51.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.83203125" customWidth="1"/>
+    <col min="7" max="8" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.83203125" customWidth="1"/>
+    <col min="10" max="10" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.83203125" customWidth="1"/>
+    <col min="12" max="12" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="3.83203125" customWidth="1"/>
+    <col min="15" max="15" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="3.83203125" customWidth="1"/>
+    <col min="17" max="17" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B1" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="R3" s="7"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="R4" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" s="12"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="M5" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="N5" s="12"/>
+      <c r="O5" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="P5" s="12"/>
+      <c r="Q5" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="R5" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B6" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="19">
+        <f>'Series A'!C7</f>
+        <v>3600000</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="Q7" s="2">
+        <f>C7</f>
+        <v>3600000</v>
+      </c>
+      <c r="R7" s="3">
+        <f>Q7/$C$47</f>
+        <v>0.15648298146475273</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="19">
+        <f>'Series A'!C8</f>
+        <v>3600000</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="Q8" s="2">
+        <f>C8</f>
+        <v>3600000</v>
+      </c>
+      <c r="R8" s="3">
+        <f>Q8/$C$47</f>
+        <v>0.15648298146475273</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="19">
+        <f>'Series A'!C9</f>
+        <v>592500</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="Q9" s="2">
+        <f>C9</f>
+        <v>592500</v>
+      </c>
+      <c r="R9" s="3">
+        <f>Q9/$C$47</f>
+        <v>2.5754490699407218E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="19">
+        <f>'Series A'!C10</f>
+        <v>592500</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="O10" s="2"/>
+      <c r="Q10" s="2">
+        <f>C10</f>
+        <v>592500</v>
+      </c>
+      <c r="R10" s="3">
+        <f>Q10/$C$47</f>
+        <v>2.5754490699407218E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="19">
+        <f>'Series A'!C11</f>
+        <v>222187</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="Q11" s="2">
+        <f>C11</f>
+        <v>222187</v>
+      </c>
+      <c r="R11" s="3">
+        <f>Q11/$C$47</f>
+        <v>9.6579122785302816E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="19">
+        <f>'Series A'!C12</f>
+        <v>285000</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="Q12" s="2">
+        <f>C12</f>
+        <v>285000</v>
+      </c>
+      <c r="R12" s="3">
+        <f>Q12/$C$47</f>
+        <v>1.2388236032626256E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="19">
+        <f>'Series A'!C13</f>
+        <v>285000</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="O13" s="2"/>
+      <c r="Q13" s="2">
+        <f>C13</f>
+        <v>285000</v>
+      </c>
+      <c r="R13" s="3">
+        <f>Q13/$C$47</f>
+        <v>1.2388236032626256E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="19">
+        <f>'Series A'!C14</f>
+        <v>112400</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="O14" s="2"/>
+      <c r="Q14" s="2">
+        <f>C14</f>
+        <v>112400</v>
+      </c>
+      <c r="R14" s="3">
+        <f>Q14/$C$47</f>
+        <v>4.8857464212883903E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>85</v>
+      </c>
+      <c r="C15" s="19">
+        <f>'Series A'!C15</f>
+        <v>385571</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="Q15" s="2">
+        <f>C15</f>
+        <v>385571</v>
+      </c>
+      <c r="R15" s="3">
+        <f>Q15/$C$47</f>
+        <v>1.675980545731838E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="19">
+        <f>'Series A'!C16</f>
+        <v>65105</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="J16" s="19">
+        <f>'Series A'!J16</f>
+        <v>1717836.4891538464</v>
+      </c>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="O16" s="2">
+        <f>$C$48</f>
+        <v>1610398.764397023</v>
+      </c>
+      <c r="Q16" s="2">
+        <f>C16+J16+O16</f>
+        <v>3393340.2535508694</v>
+      </c>
+      <c r="R16" s="3">
+        <f>Q16/$C$47</f>
+        <v>0.14749999999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B17" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" s="4">
+        <f>SUM(C7:C16)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="4">
+        <f>SUM(J7:J16)</f>
+        <v>1717836.4891538464</v>
+      </c>
+      <c r="K17" s="1"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="4">
+        <f>SUM(O7:O16)</f>
+        <v>1610398.764397023</v>
+      </c>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="4">
+        <f>SUM(Q7:Q16)</f>
+        <v>13068498.253550868</v>
+      </c>
+      <c r="R17" s="5">
+        <f>Q17/$C$47</f>
+        <v>0.56805488055070941</v>
+      </c>
+    </row>
+    <row r="18" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="3"/>
+    </row>
+    <row r="19" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="O19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="3"/>
+    </row>
+    <row r="20" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="19">
+        <f>'Series A'!D20</f>
+        <v>8000000</v>
+      </c>
+      <c r="E20" s="19">
+        <f>'Series A'!E20</f>
+        <v>1558442.08</v>
+      </c>
+      <c r="G20" s="19">
+        <f>'Series A'!G20</f>
+        <v>5000000</v>
+      </c>
+      <c r="H20" s="19">
+        <f>'Series A'!H20</f>
+        <v>1114338.430721154</v>
+      </c>
+      <c r="J20" s="2"/>
+      <c r="L20" s="2">
+        <f>$C$50</f>
+        <v>3750000</v>
+      </c>
+      <c r="M20" s="2">
+        <f>L20/$C$44</f>
+        <v>445735.3722884616</v>
+      </c>
+      <c r="O20" s="2"/>
+      <c r="Q20" s="2">
+        <f>E20+H20+M20</f>
+        <v>3118515.8830096158</v>
+      </c>
+      <c r="R20" s="3">
+        <f>Q20/$C$47</f>
+        <v>0.13555407308848075</v>
+      </c>
+    </row>
+    <row r="21" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B21" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="19">
+        <f>'Series A'!D21</f>
+        <v>250000</v>
+      </c>
+      <c r="E21" s="19">
+        <f>'Series A'!E21</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="O21" s="2"/>
+      <c r="Q21" s="2">
+        <f>E21</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="R21" s="3">
+        <f>Q21/$C$47</f>
+        <v>2.1169241590150234E-3</v>
+      </c>
+    </row>
+    <row r="22" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="19">
+        <f>'Series A'!D22</f>
+        <v>300000</v>
+      </c>
+      <c r="E22" s="19">
+        <f>'Series A'!E22</f>
+        <v>58441.578000000001</v>
+      </c>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="O22" s="2"/>
+      <c r="Q22" s="2">
+        <f>E22</f>
+        <v>58441.578000000001</v>
+      </c>
+      <c r="R22" s="3">
+        <f>Q22/$C$47</f>
+        <v>2.5403089908180281E-3</v>
+      </c>
+    </row>
+    <row r="23" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" s="19">
+        <f>'Series A'!D23</f>
+        <v>250000</v>
+      </c>
+      <c r="E23" s="19">
+        <f>'Series A'!E23</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
+      <c r="O23" s="2"/>
+      <c r="Q23" s="2">
+        <f>E23</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="R23" s="3">
+        <f>Q23/$C$47</f>
+        <v>2.1169241590150234E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="19">
+        <f>'Series A'!D24</f>
+        <v>212500</v>
+      </c>
+      <c r="E24" s="19">
+        <f>'Series A'!E24</f>
+        <v>41396.117749999998</v>
+      </c>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+      <c r="O24" s="2"/>
+      <c r="Q24" s="2">
+        <f>E24</f>
+        <v>41396.117749999998</v>
+      </c>
+      <c r="R24" s="3">
+        <f>Q24/$C$47</f>
+        <v>1.7993855351627697E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B25" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="19">
+        <f>'Series A'!D25</f>
+        <v>250000</v>
+      </c>
+      <c r="E25" s="19">
+        <f>'Series A'!E25</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
+      <c r="O25" s="2"/>
+      <c r="Q25" s="2">
+        <f>E25</f>
+        <v>48701.315000000002</v>
+      </c>
+      <c r="R25" s="3">
+        <f>Q25/$C$47</f>
+        <v>2.1169241590150234E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>88</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="19">
+        <f>'Series A'!D26</f>
+        <v>562500</v>
+      </c>
+      <c r="E26" s="19">
+        <f>'Series A'!E26</f>
+        <v>109577.95875000001</v>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
+      <c r="O26" s="2"/>
+      <c r="Q26" s="2">
+        <f>E26</f>
+        <v>109577.95875000001</v>
+      </c>
+      <c r="R26" s="3">
+        <f>Q26/$C$47</f>
+        <v>4.7630793577838025E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B27" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="G27" s="19">
+        <f>'Series A'!G27</f>
+        <v>12000000</v>
+      </c>
+      <c r="H27" s="19">
+        <f>'Series A'!H27</f>
+        <v>2674412.2337307697</v>
+      </c>
+      <c r="J27" s="2"/>
+      <c r="L27" s="2">
+        <f>$C$49</f>
+        <v>9000000</v>
+      </c>
+      <c r="M27" s="2">
+        <f>L27/$C$44</f>
+        <v>1069764.8934923077</v>
+      </c>
+      <c r="O27" s="2"/>
+      <c r="Q27" s="2">
+        <f>H27+M27</f>
+        <v>3744177.1272230772</v>
+      </c>
+      <c r="R27" s="3">
+        <f>Q27/$C$47</f>
+        <v>0.16274999999999998</v>
+      </c>
+    </row>
+    <row r="28" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B28" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="G28" s="19">
+        <f>'Series A'!G28</f>
+        <v>3000000</v>
+      </c>
+      <c r="H28" s="19">
+        <f>'Series A'!H28</f>
+        <v>668603.05843269243</v>
+      </c>
+      <c r="J28" s="2"/>
+      <c r="L28" s="2">
+        <f>$C$51</f>
+        <v>2250000</v>
+      </c>
+      <c r="M28" s="2">
+        <f>L28/$C$44</f>
+        <v>267441.22337307694</v>
+      </c>
+      <c r="O28" s="2"/>
+      <c r="Q28" s="2">
+        <f>H28+M28</f>
+        <v>936044.28180576931</v>
+      </c>
+      <c r="R28" s="3">
+        <f>Q28/$C$47</f>
+        <v>4.0687499999999995E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B29" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="J29" s="2"/>
+      <c r="L29" s="2">
+        <f>$C$38</f>
+        <v>15000000</v>
+      </c>
+      <c r="M29" s="2">
+        <f>L29/$C$44</f>
+        <v>1782941.4891538464</v>
+      </c>
+      <c r="O29" s="2"/>
+      <c r="Q29" s="2">
+        <f>M29</f>
+        <v>1782941.4891538464</v>
+      </c>
+      <c r="R29" s="3">
+        <f>Q29/$C$47</f>
+        <v>7.7499999999999986E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="J30" s="2"/>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
+      <c r="O30" s="2"/>
+      <c r="Q30" s="2"/>
+      <c r="R30" s="3"/>
+    </row>
+    <row r="31" spans="2:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="16">
+        <f>SUM(C7:C16)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D31" s="16">
+        <f>SUM(D20:D26)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E31" s="16">
+        <f>SUM(E20:E26)</f>
+        <v>1913961.6794999999</v>
+      </c>
+      <c r="F31" s="13"/>
+      <c r="G31" s="16">
+        <f>SUM(G20:G28)</f>
+        <v>20000000</v>
+      </c>
+      <c r="H31" s="16">
+        <f>SUM(H20:H28)</f>
+        <v>4457353.7228846159</v>
+      </c>
+      <c r="I31" s="13"/>
+      <c r="J31" s="16">
+        <f>J16</f>
+        <v>1717836.4891538464</v>
+      </c>
+      <c r="K31" s="13"/>
+      <c r="L31" s="16">
+        <f>SUM(L20:L29)</f>
+        <v>30000000</v>
+      </c>
+      <c r="M31" s="16">
+        <f>SUM(M20:M29)</f>
+        <v>3565882.9783076923</v>
+      </c>
+      <c r="N31" s="13"/>
+      <c r="O31" s="16">
+        <f>O16</f>
+        <v>1610398.764397023</v>
+      </c>
+      <c r="P31" s="13"/>
+      <c r="Q31" s="16">
+        <f>C31+E31+H31+J31+M31+O31</f>
+        <v>23005696.634243179</v>
+      </c>
+      <c r="R31" s="17">
+        <f>Q31/$C$47</f>
+        <v>0.99999999999999989</v>
+      </c>
+    </row>
+    <row r="32" spans="2:18" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="33" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B33" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="E33" s="21">
+        <f>'Series A'!E32</f>
+        <v>5.1333316153783528</v>
+      </c>
+      <c r="H33" s="21">
+        <f>'Series A'!H32</f>
+        <v>4.48696721045886</v>
+      </c>
+      <c r="M33" s="18">
+        <f>$C$44</f>
+        <v>8.4130635196103629</v>
+      </c>
+    </row>
+    <row r="34" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E34" s="19">
+        <f>'Series A'!E33</f>
+        <v>50000000</v>
+      </c>
+      <c r="H34" s="19">
+        <f>'Series A'!H33</f>
+        <v>60000000</v>
+      </c>
+      <c r="M34" s="2">
+        <f>$C$36</f>
+        <v>150000000</v>
+      </c>
+    </row>
+    <row r="35" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B35" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="36" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B36" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="14">
+        <v>150000000</v>
+      </c>
+    </row>
+    <row r="37" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B37" t="s">
+        <v>75</v>
+      </c>
+      <c r="C37" s="14">
+        <v>30000000</v>
+      </c>
+    </row>
+    <row r="38" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B38" t="s">
+        <v>101</v>
+      </c>
+      <c r="C38" s="14">
+        <v>15000000</v>
+      </c>
+    </row>
+    <row r="39" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>102</v>
+      </c>
+      <c r="C39" s="2">
+        <f>C37-C38</f>
+        <v>15000000</v>
+      </c>
+    </row>
+    <row r="40" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>103</v>
+      </c>
+      <c r="C40" s="15">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B41" t="s">
+        <v>73</v>
+      </c>
+      <c r="C41" s="2">
+        <f>C36+C37</f>
+        <v>180000000</v>
+      </c>
+    </row>
+    <row r="42" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>104</v>
+      </c>
+      <c r="C42" s="19">
+        <f>'Series A'!C49</f>
+        <v>17829414.891538464</v>
+      </c>
+    </row>
+    <row r="43" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
+        <v>105</v>
+      </c>
+      <c r="C43" s="19">
+        <f>'Series A'!L16</f>
+        <v>1782941.4891538464</v>
+      </c>
+    </row>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
+        <v>106</v>
+      </c>
+      <c r="C44" s="18">
+        <f>C36/C42</f>
+        <v>8.4130635196103629</v>
+      </c>
+    </row>
+    <row r="45" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
+        <v>107</v>
+      </c>
+      <c r="C45" s="2">
+        <f>C37/C44</f>
+        <v>3565882.9783076928</v>
+      </c>
+    </row>
+    <row r="46" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B46" t="s">
+        <v>108</v>
+      </c>
+      <c r="C46" s="2">
+        <f>C42+C45</f>
+        <v>21395297.869846158</v>
+      </c>
+    </row>
+    <row r="47" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B47" t="s">
+        <v>109</v>
+      </c>
+      <c r="C47" s="2">
+        <f>C46/(1-C40)</f>
+        <v>23005696.634243183</v>
+      </c>
+    </row>
+    <row r="48" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B48" t="s">
+        <v>110</v>
+      </c>
+      <c r="C48" s="2">
+        <f>C40*C47</f>
+        <v>1610398.764397023</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B49" t="s">
+        <v>111</v>
+      </c>
+      <c r="C49" s="19">
+        <f>C39*'Series A'!C38/'Series A'!C37</f>
+        <v>9000000</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B50" t="s">
+        <v>112</v>
+      </c>
+      <c r="C50" s="19">
+        <f>C39*'Series A'!C39/'Series A'!C37</f>
+        <v>3750000</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B51" t="s">
+        <v>113</v>
+      </c>
+      <c r="C51" s="19">
+        <f>C39*'Series A'!C40/'Series A'!C37</f>
+        <v>2250000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checkpoint: Rebuilt all 4 sheets: Sidekick Cap Table, SAFE Investments, Series A, Series B
</commit_message>
<xml_diff>
--- a/runs/resume/models/model.xlsx
+++ b/runs/resume/models/model.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2B8674A8-8D31-A842-80F7-DC0C9C95F142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF3CCEAB-432D-D145-A60E-DD145A710A52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sidekick Cap Table" sheetId="19" r:id="rId1"/>
-    <sheet name="SAFE Investments" sheetId="20" r:id="rId2"/>
-    <sheet name="Series A" sheetId="24" r:id="rId3"/>
-    <sheet name="Series B" sheetId="25" r:id="rId4"/>
+    <sheet name="Sidekick Cap Table" sheetId="27" r:id="rId1"/>
+    <sheet name="SAFE Investments" sheetId="28" r:id="rId2"/>
+    <sheet name="Series A" sheetId="29" r:id="rId3"/>
+    <sheet name="Series B" sheetId="30" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="114">
   <si>
     <t>Total</t>
   </si>
@@ -338,9 +338,6 @@
     <t>Total Series A Shares</t>
   </si>
   <si>
-    <t>Check (Investments = Total Raised)</t>
-  </si>
-  <si>
     <t>Other Series B Investment</t>
   </si>
   <si>
@@ -353,9 +350,6 @@
     <t>Post-A Total FD Shares</t>
   </si>
   <si>
-    <t>Post-A ESOP Available</t>
-  </si>
-  <si>
     <t>Series B Price per Share</t>
   </si>
   <si>
@@ -377,13 +371,13 @@
     <t>Accomplice Pro Rata B Investment</t>
   </si>
   <si>
-    <t>Other A Investors Pro Rata B Investment</t>
-  </si>
-  <si>
     <t>SIDEKICK (THINK MORE SECURITY) &amp; 1011/ACCOMPLICE SERIES B</t>
   </si>
   <si>
     <t>Other Series B Investors</t>
+  </si>
+  <si>
+    <t>Other A Pro Rata B Investment</t>
   </si>
 </sst>
 </file>
@@ -530,18 +524,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color rgb="FF0000FF"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -924,35 +919,32 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="18" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="18" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="19" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="19" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1345,17 +1337,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA63D99-0A1B-7A4C-810F-F1C88706AF91}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDB9267C-205A-5A49-BD8C-9FE6B1CFC72F}">
   <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.83203125" customWidth="1"/>
     <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -1371,26 +1363,26 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="8"/>
-      <c r="B2" s="8" t="s">
+      <c r="A2" s="17"/>
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="17" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1398,16 +1390,16 @@
       <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="3">
         <v>3600000</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2">
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3">
         <v>3600000</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="4">
         <v>0.36959987630724139</v>
       </c>
     </row>
@@ -1415,16 +1407,16 @@
       <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
         <v>3600000</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2">
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3">
         <v>3600000</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="4">
         <v>0.36959987630724139</v>
       </c>
     </row>
@@ -1432,16 +1424,16 @@
       <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="3">
         <v>222187</v>
       </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2">
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3">
         <v>222187</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="4">
         <v>2.28111910325214E-2</v>
       </c>
     </row>
@@ -1449,16 +1441,16 @@
       <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="3">
         <v>592500</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2">
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3">
         <v>592500</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="4">
         <v>6.0829979642233481E-2</v>
       </c>
     </row>
@@ -1466,16 +1458,16 @@
       <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="3">
         <v>592500</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2">
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3">
         <v>592500</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="4">
         <v>6.0829979642233481E-2</v>
       </c>
     </row>
@@ -1483,18 +1475,18 @@
       <c r="B8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="3">
         <v>13500</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="3">
         <v>98900</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2">
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3">
         <v>112400</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="4">
         <v>1.1539729471370537E-2</v>
       </c>
     </row>
@@ -1502,16 +1494,16 @@
       <c r="B9" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="3">
         <v>9000</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2">
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3">
         <v>9000</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="4">
         <v>9.2399969076810353E-4</v>
       </c>
     </row>
@@ -1519,16 +1511,16 @@
       <c r="B10" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2">
+      <c r="C10" s="3"/>
+      <c r="D10" s="3">
         <v>95000</v>
       </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2">
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3">
         <v>95000</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="4">
         <v>9.7533300692188695E-3</v>
       </c>
     </row>
@@ -1536,16 +1528,16 @@
       <c r="B11" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2">
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3">
         <v>25000</v>
       </c>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2">
+      <c r="F11" s="3"/>
+      <c r="G11" s="3">
         <v>25000</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="4">
         <v>2.5666658076891765E-3</v>
       </c>
     </row>
@@ -1553,16 +1545,16 @@
       <c r="B12" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2">
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3">
         <v>41562</v>
       </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2">
+      <c r="F12" s="3"/>
+      <c r="G12" s="3">
         <v>41562</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="4">
         <v>4.2670305719671019E-3</v>
       </c>
     </row>
@@ -1570,16 +1562,16 @@
       <c r="B13" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2">
+      <c r="C13" s="3"/>
+      <c r="D13" s="3">
         <v>285000</v>
       </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2">
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3">
         <v>285000</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="4">
         <v>2.925999020765661E-2</v>
       </c>
     </row>
@@ -1587,16 +1579,16 @@
       <c r="B14" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2">
+      <c r="C14" s="3"/>
+      <c r="D14" s="3">
         <v>50000</v>
       </c>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2">
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3">
         <v>50000</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="4">
         <v>5.133331615378353E-3</v>
       </c>
     </row>
@@ -1604,16 +1596,16 @@
       <c r="B15" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2">
+      <c r="C15" s="3"/>
+      <c r="D15" s="3">
         <v>285000</v>
       </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2">
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3">
         <v>285000</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="4">
         <v>2.925999020765661E-2</v>
       </c>
     </row>
@@ -1621,16 +1613,16 @@
       <c r="B16" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2">
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3">
         <v>96186</v>
       </c>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2">
+      <c r="F16" s="3"/>
+      <c r="G16" s="3">
         <v>96186</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="4">
         <v>9.8750926951356455E-3</v>
       </c>
     </row>
@@ -1638,16 +1630,16 @@
       <c r="B17" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2">
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3">
         <v>48095</v>
       </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2">
+      <c r="F17" s="3"/>
+      <c r="G17" s="3">
         <v>48095</v>
       </c>
-      <c r="H17" s="3">
+      <c r="H17" s="4">
         <v>4.9377516808324371E-3</v>
       </c>
     </row>
@@ -1655,16 +1647,16 @@
       <c r="B18" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2">
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3">
         <v>12395</v>
       </c>
-      <c r="G18" s="2">
+      <c r="G18" s="3">
         <v>12395</v>
       </c>
-      <c r="H18" s="3">
+      <c r="H18" s="4">
         <v>1.2725529074522936E-3</v>
       </c>
     </row>
@@ -1672,16 +1664,16 @@
       <c r="B19" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2">
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3">
         <v>8333</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G19" s="3">
         <v>8333</v>
       </c>
-      <c r="H19" s="3">
+      <c r="H19" s="4">
         <v>8.5552104701895626E-4</v>
       </c>
     </row>
@@ -1689,40 +1681,40 @@
       <c r="B20" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2">
+      <c r="C20" s="3"/>
+      <c r="D20" s="3">
         <v>65105</v>
       </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2">
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3">
         <v>65105</v>
       </c>
-      <c r="H20" s="3">
+      <c r="H20" s="4">
         <v>6.6841110963841528E-3</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9" t="s">
+      <c r="A21" s="8"/>
+      <c r="B21" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="11">
         <v>8629687</v>
       </c>
-      <c r="D21" s="10">
+      <c r="D21" s="11">
         <v>879005</v>
       </c>
-      <c r="E21" s="10">
+      <c r="E21" s="11">
         <v>210843</v>
       </c>
-      <c r="F21" s="10">
+      <c r="F21" s="11">
         <v>20728</v>
       </c>
-      <c r="G21" s="10">
+      <c r="G21" s="11">
         <v>9740263</v>
       </c>
-      <c r="H21" s="11"/>
+      <c r="H21" s="12"/>
     </row>
     <row r="22" spans="1:8" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
@@ -1731,7 +1723,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DEFA1E8-9CBB-4243-8159-522C32655D43}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84918C69-B8E7-CE44-AE24-F1E96B5F3BD7}">
   <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1743,15 +1735,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="8"/>
-      <c r="B1" s="8" t="s">
+      <c r="A1" s="17"/>
+      <c r="B1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8" t="s">
+      <c r="D1" s="17"/>
+      <c r="E1" s="17" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1759,7 +1751,7 @@
       <c r="B2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="3">
         <v>25000</v>
       </c>
       <c r="E2" t="s">
@@ -1770,7 +1762,7 @@
       <c r="B3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="3">
         <v>25000</v>
       </c>
     </row>
@@ -1778,7 +1770,7 @@
       <c r="B4" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
         <v>137170.75</v>
       </c>
     </row>
@@ -1786,7 +1778,7 @@
       <c r="B5" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="3">
         <v>3846829.25</v>
       </c>
     </row>
@@ -1794,7 +1786,7 @@
       <c r="B6" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="3">
         <v>16566</v>
       </c>
       <c r="E6" t="s">
@@ -1805,7 +1797,7 @@
       <c r="B7" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="3">
         <v>250000</v>
       </c>
     </row>
@@ -1813,7 +1805,7 @@
       <c r="B8" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="3">
         <v>100000</v>
       </c>
     </row>
@@ -1821,7 +1813,7 @@
       <c r="B9" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="3">
         <v>300000</v>
       </c>
       <c r="E9" t="s">
@@ -1832,7 +1824,7 @@
       <c r="B10" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="3">
         <v>37500</v>
       </c>
       <c r="E10" t="s">
@@ -1843,7 +1835,7 @@
       <c r="B11" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="3">
         <v>250000</v>
       </c>
     </row>
@@ -1851,7 +1843,7 @@
       <c r="B12" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="3">
         <v>100000</v>
       </c>
     </row>
@@ -1859,7 +1851,7 @@
       <c r="B13" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="3">
         <v>41164</v>
       </c>
       <c r="E13" t="s">
@@ -1870,7 +1862,7 @@
       <c r="B14" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="3">
         <v>2328778</v>
       </c>
       <c r="E14" t="s">
@@ -1881,7 +1873,7 @@
       <c r="B15" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="3">
         <v>1506000</v>
       </c>
       <c r="E15" t="s">
@@ -1892,7 +1884,7 @@
       <c r="B16" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="3">
         <v>50000</v>
       </c>
     </row>
@@ -1900,7 +1892,7 @@
       <c r="B17" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="3">
         <v>212500</v>
       </c>
       <c r="E17" t="s">
@@ -1911,7 +1903,7 @@
       <c r="B18" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="3">
         <v>25000</v>
       </c>
     </row>
@@ -1919,7 +1911,7 @@
       <c r="B19" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="3">
         <v>61746</v>
       </c>
       <c r="E19" t="s">
@@ -1930,7 +1922,7 @@
       <c r="B20" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="3">
         <v>100000</v>
       </c>
     </row>
@@ -1938,7 +1930,7 @@
       <c r="B21" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="3">
         <v>100000</v>
       </c>
     </row>
@@ -1946,7 +1938,7 @@
       <c r="B22" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="3">
         <v>61746</v>
       </c>
       <c r="E22" t="s">
@@ -1957,7 +1949,7 @@
       <c r="B23" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23" s="3">
         <v>250000</v>
       </c>
       <c r="E23" t="s">
@@ -1965,15 +1957,15 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="9"/>
-      <c r="B24" s="9" t="s">
+      <c r="A24" s="8"/>
+      <c r="B24" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C24" s="10">
+      <c r="C24" s="11">
         <v>9825000</v>
       </c>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
     </row>
     <row r="25" spans="1:5" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
@@ -1982,12 +1974,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BDD7B37-73DF-F641-9F36-44DBA8C4C9E2}">
-  <dimension ref="A1:M53"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C93607-5037-6844-A950-0B90DDD4B1BD}">
+  <dimension ref="A1:M52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.83203125" customWidth="1"/>
-    <col min="2" max="2" width="51.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
@@ -1996,12 +1988,12 @@
     <col min="9" max="9" width="3.83203125" customWidth="1"/>
     <col min="10" max="10" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="3.83203125" customWidth="1"/>
-    <col min="12" max="12" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="2" t="s">
         <v>84</v>
       </c>
     </row>
@@ -2062,33 +2054,33 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="12"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12" t="s">
+      <c r="A5" s="18"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12" t="s">
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="H5" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12" t="s">
+      <c r="I5" s="18"/>
+      <c r="J5" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12" t="s">
+      <c r="K5" s="18"/>
+      <c r="L5" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="M5" s="12" t="s">
+      <c r="M5" s="18" t="s">
         <v>64</v>
       </c>
     </row>
@@ -2101,20 +2093,20 @@
       <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="14">
         <f>'Sidekick Cap Table'!G3</f>
         <v>3600000</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="L7" s="2">
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="L7" s="3">
         <f>C7</f>
         <v>3600000</v>
       </c>
-      <c r="M7" s="3">
+      <c r="M7" s="4">
         <f>L7/$C$49</f>
         <v>0.2019135244706487</v>
       </c>
@@ -2123,20 +2115,20 @@
       <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="14">
         <f>'Sidekick Cap Table'!G4</f>
         <v>3600000</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="L8" s="2">
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="L8" s="3">
         <f>C8</f>
         <v>3600000</v>
       </c>
-      <c r="M8" s="3">
+      <c r="M8" s="4">
         <f>L8/$C$49</f>
         <v>0.2019135244706487</v>
       </c>
@@ -2145,20 +2137,20 @@
       <c r="B9" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="14">
         <f>'Sidekick Cap Table'!G6</f>
         <v>592500</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="L9" s="2">
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="L9" s="3">
         <f>C9</f>
         <v>592500</v>
       </c>
-      <c r="M9" s="3">
+      <c r="M9" s="4">
         <f>L9/$C$49</f>
         <v>3.3231600902460932E-2</v>
       </c>
@@ -2167,20 +2159,20 @@
       <c r="B10" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="19">
+      <c r="C10" s="14">
         <f>'Sidekick Cap Table'!G7</f>
         <v>592500</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="L10" s="2">
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="L10" s="3">
         <f>C10</f>
         <v>592500</v>
       </c>
-      <c r="M10" s="3">
+      <c r="M10" s="4">
         <f>L10/$C$49</f>
         <v>3.3231600902460932E-2</v>
       </c>
@@ -2189,20 +2181,20 @@
       <c r="B11" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="14">
         <f>'Sidekick Cap Table'!G5</f>
         <v>222187</v>
       </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="L11" s="2">
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="L11" s="3">
         <f>C11</f>
         <v>222187</v>
       </c>
-      <c r="M11" s="3">
+      <c r="M11" s="4">
         <f>L11/$C$49</f>
         <v>1.2461822294877785E-2</v>
       </c>
@@ -2211,20 +2203,20 @@
       <c r="B12" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="14">
         <f>'Sidekick Cap Table'!G13</f>
         <v>285000</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="L12" s="2">
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="L12" s="3">
         <f>C12</f>
         <v>285000</v>
       </c>
-      <c r="M12" s="3">
+      <c r="M12" s="4">
         <f>L12/$C$49</f>
         <v>1.598482068725969E-2</v>
       </c>
@@ -2233,20 +2225,20 @@
       <c r="B13" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="14">
         <f>'Sidekick Cap Table'!G15</f>
         <v>285000</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="L13" s="2">
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="L13" s="3">
         <f>C13</f>
         <v>285000</v>
       </c>
-      <c r="M13" s="3">
+      <c r="M13" s="4">
         <f>L13/$C$49</f>
         <v>1.598482068725969E-2</v>
       </c>
@@ -2255,20 +2247,20 @@
       <c r="B14" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="14">
         <f>'Sidekick Cap Table'!G8</f>
         <v>112400</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="L14" s="2">
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="L14" s="3">
         <f>C14</f>
         <v>112400</v>
       </c>
-      <c r="M14" s="3">
+      <c r="M14" s="4">
         <f>L14/$C$49</f>
         <v>6.3041889306946989E-3</v>
       </c>
@@ -2277,20 +2269,20 @@
       <c r="B15" t="s">
         <v>85</v>
       </c>
-      <c r="C15" s="19">
+      <c r="C15" s="14">
         <f>'Sidekick Cap Table'!G9+'Sidekick Cap Table'!G10+'Sidekick Cap Table'!G11+'Sidekick Cap Table'!G12+'Sidekick Cap Table'!G14+'Sidekick Cap Table'!G16+'Sidekick Cap Table'!G17+'Sidekick Cap Table'!G18+'Sidekick Cap Table'!G19</f>
         <v>385571</v>
       </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="L15" s="2">
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="L15" s="3">
         <f>C15</f>
         <v>385571</v>
       </c>
-      <c r="M15" s="3">
+      <c r="M15" s="4">
         <f>L15/$C$49</f>
         <v>2.1625555428797915E-2</v>
       </c>
@@ -2299,23 +2291,23 @@
       <c r="B16" t="s">
         <v>86</v>
       </c>
-      <c r="C16" s="19">
+      <c r="C16" s="14">
         <f>'Sidekick Cap Table'!G20</f>
         <v>65105</v>
       </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="J16" s="2">
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="J16" s="3">
         <f>$C$52</f>
         <v>1717836.4891538464</v>
       </c>
-      <c r="L16" s="2">
+      <c r="L16" s="3">
         <f>C16+J16</f>
         <v>1782941.4891538464</v>
       </c>
-      <c r="M16" s="3">
+      <c r="M16" s="4">
         <f>L16/$C$49</f>
         <v>0.1</v>
       </c>
@@ -2324,80 +2316,80 @@
       <c r="B17" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="5">
         <f>SUM(C7:C16)</f>
         <v>9740263</v>
       </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="4">
+      <c r="J17" s="5">
         <f>SUM(J7:J16)</f>
         <v>1717836.4891538464</v>
       </c>
       <c r="K17" s="1"/>
-      <c r="L17" s="4">
+      <c r="L17" s="5">
         <f>SUM(L7:L16)</f>
         <v>11458099.489153847</v>
       </c>
-      <c r="M17" s="5">
+      <c r="M17" s="6">
         <f>L17/$C$49</f>
         <v>0.6426514587751091</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="4"/>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="4"/>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>87</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="19">
+      <c r="C20" s="3"/>
+      <c r="D20" s="14">
         <f>'SAFE Investments'!C4+'SAFE Investments'!C5+'SAFE Investments'!C6+'SAFE Investments'!C13+'SAFE Investments'!C14+'SAFE Investments'!C15+'SAFE Investments'!C19+'SAFE Investments'!C22</f>
         <v>8000000</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="3">
         <f>D20/$C$47</f>
         <v>1558442.08</v>
       </c>
-      <c r="G20" s="2">
+      <c r="G20" s="3">
         <f>$C$39</f>
         <v>5000000</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="3">
         <f>G20/$C$50</f>
         <v>1114338.430721154</v>
       </c>
-      <c r="J20" s="2"/>
-      <c r="L20" s="2">
+      <c r="J20" s="3"/>
+      <c r="L20" s="3">
         <f>E20+H20</f>
         <v>2672780.510721154</v>
       </c>
-      <c r="M20" s="3">
+      <c r="M20" s="4">
         <f>L20/$C$49</f>
         <v>0.14990848140449131</v>
       </c>
@@ -2406,23 +2398,23 @@
       <c r="B21" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="19">
+      <c r="C21" s="3"/>
+      <c r="D21" s="14">
         <f>'SAFE Investments'!C7</f>
         <v>250000</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="3">
         <f>D21/$C$47</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="L21" s="2">
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="L21" s="3">
         <f>E21</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="M21" s="3">
+      <c r="M21" s="4">
         <f>L21/$C$49</f>
         <v>2.7315150438903531E-3</v>
       </c>
@@ -2431,23 +2423,23 @@
       <c r="B22" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="19">
+      <c r="C22" s="3"/>
+      <c r="D22" s="14">
         <f>'SAFE Investments'!C9</f>
         <v>300000</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="3">
         <f>D22/$C$47</f>
         <v>58441.578000000001</v>
       </c>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="L22" s="2">
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="L22" s="3">
         <f>E22</f>
         <v>58441.578000000001</v>
       </c>
-      <c r="M22" s="3">
+      <c r="M22" s="4">
         <f>L22/$C$49</f>
         <v>3.2778180526684235E-3</v>
       </c>
@@ -2456,23 +2448,23 @@
       <c r="B23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="19">
+      <c r="C23" s="3"/>
+      <c r="D23" s="14">
         <f>'SAFE Investments'!C11</f>
         <v>250000</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="3">
         <f>D23/$C$47</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="L23" s="2">
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="L23" s="3">
         <f>E23</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="M23" s="3">
+      <c r="M23" s="4">
         <f>L23/$C$49</f>
         <v>2.7315150438903531E-3</v>
       </c>
@@ -2481,23 +2473,23 @@
       <c r="B24" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="19">
+      <c r="C24" s="3"/>
+      <c r="D24" s="14">
         <f>'SAFE Investments'!C17</f>
         <v>212500</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="3">
         <f>D24/$C$47</f>
         <v>41396.117749999998</v>
       </c>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="L24" s="2">
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="L24" s="3">
         <f>E24</f>
         <v>41396.117749999998</v>
       </c>
-      <c r="M24" s="3">
+      <c r="M24" s="4">
         <f>L24/$C$49</f>
         <v>2.3217877873068001E-3</v>
       </c>
@@ -2506,23 +2498,23 @@
       <c r="B25" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="19">
+      <c r="C25" s="3"/>
+      <c r="D25" s="14">
         <f>'SAFE Investments'!C23</f>
         <v>250000</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="3">
         <f>D25/$C$47</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="L25" s="2">
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="L25" s="3">
         <f>E25</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="M25" s="3">
+      <c r="M25" s="4">
         <f>L25/$C$49</f>
         <v>2.7315150438903531E-3</v>
       </c>
@@ -2531,23 +2523,23 @@
       <c r="B26" t="s">
         <v>88</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="19">
+      <c r="C26" s="3"/>
+      <c r="D26" s="14">
         <f>'SAFE Investments'!C2+'SAFE Investments'!C3+'SAFE Investments'!C8+'SAFE Investments'!C10+'SAFE Investments'!C12+'SAFE Investments'!C16+'SAFE Investments'!C18+'SAFE Investments'!C20+'SAFE Investments'!C21</f>
         <v>562500</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="3">
         <f>D26/$C$47</f>
         <v>109577.95875000001</v>
       </c>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="L26" s="2">
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="L26" s="3">
         <f>E26</f>
         <v>109577.95875000001</v>
       </c>
-      <c r="M26" s="3">
+      <c r="M26" s="4">
         <f>L26/$C$49</f>
         <v>6.1459088487532945E-3</v>
       </c>
@@ -2556,23 +2548,23 @@
       <c r="B27" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="G27" s="2">
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="G27" s="3">
         <f>$C$38</f>
         <v>12000000</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="3">
         <f>G27/$C$50</f>
         <v>2674412.2337307697</v>
       </c>
-      <c r="J27" s="2"/>
-      <c r="L27" s="2">
+      <c r="J27" s="3"/>
+      <c r="L27" s="3">
         <f>H27</f>
         <v>2674412.2337307697</v>
       </c>
-      <c r="M27" s="3">
+      <c r="M27" s="4">
         <f>L27/$C$49</f>
         <v>0.15000000000000002</v>
       </c>
@@ -2581,73 +2573,73 @@
       <c r="B28" t="s">
         <v>69</v>
       </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="G28" s="2">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="G28" s="3">
         <f>$C$40</f>
         <v>3000000</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="3">
         <f>G28/$C$50</f>
         <v>668603.05843269243</v>
       </c>
-      <c r="J28" s="2"/>
-      <c r="L28" s="2">
+      <c r="J28" s="3"/>
+      <c r="L28" s="3">
         <f>H28</f>
         <v>668603.05843269243</v>
       </c>
-      <c r="M28" s="3">
+      <c r="M28" s="4">
         <f>L28/$C$49</f>
         <v>3.7500000000000006E-2</v>
       </c>
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="4"/>
     </row>
     <row r="30" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="11">
         <f>SUM(C7:C16)</f>
         <v>9740263</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="11">
         <f>SUM(D20:D26)</f>
         <v>9825000</v>
       </c>
-      <c r="E30" s="16">
+      <c r="E30" s="11">
         <f>SUM(E20:E26)</f>
         <v>1913961.6794999999</v>
       </c>
-      <c r="F30" s="13"/>
-      <c r="G30" s="16">
+      <c r="F30" s="8"/>
+      <c r="G30" s="11">
         <f>SUM(G20:G28)</f>
         <v>20000000</v>
       </c>
-      <c r="H30" s="16">
+      <c r="H30" s="11">
         <f>SUM(H20:H28)</f>
         <v>4457353.7228846159</v>
       </c>
-      <c r="I30" s="13"/>
-      <c r="J30" s="16">
+      <c r="I30" s="8"/>
+      <c r="J30" s="11">
         <f>J16</f>
         <v>1717836.4891538464</v>
       </c>
-      <c r="K30" s="13"/>
-      <c r="L30" s="16">
+      <c r="K30" s="8"/>
+      <c r="L30" s="11">
         <f>C30+E30+H30+J30</f>
         <v>17829414.891538464</v>
       </c>
-      <c r="M30" s="17">
+      <c r="M30" s="12">
         <f>L30/$C$49</f>
         <v>1</v>
       </c>
@@ -2657,11 +2649,11 @@
       <c r="B32" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E32" s="18">
+      <c r="E32" s="13">
         <f>$C$47</f>
         <v>5.1333316153783528</v>
       </c>
-      <c r="H32" s="18">
+      <c r="H32" s="13">
         <f>$C$50</f>
         <v>4.48696721045886</v>
       </c>
@@ -2670,11 +2662,11 @@
       <c r="B33" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="3">
         <f>$C$42</f>
         <v>50000000</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="3">
         <f>$C$36</f>
         <v>60000000</v>
       </c>
@@ -2683,11 +2675,11 @@
       <c r="B34" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="3">
         <f>$C$42</f>
         <v>50000000</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="3">
         <f>$C$41</f>
         <v>80000000</v>
       </c>
@@ -2701,7 +2693,7 @@
       <c r="B36" t="s">
         <v>72</v>
       </c>
-      <c r="C36" s="14">
+      <c r="C36" s="9">
         <v>60000000</v>
       </c>
     </row>
@@ -2709,7 +2701,7 @@
       <c r="B37" t="s">
         <v>75</v>
       </c>
-      <c r="C37" s="14">
+      <c r="C37" s="9">
         <v>20000000</v>
       </c>
     </row>
@@ -2717,7 +2709,7 @@
       <c r="B38" t="s">
         <v>76</v>
       </c>
-      <c r="C38" s="14">
+      <c r="C38" s="9">
         <v>12000000</v>
       </c>
     </row>
@@ -2725,7 +2717,7 @@
       <c r="B39" t="s">
         <v>77</v>
       </c>
-      <c r="C39" s="14">
+      <c r="C39" s="9">
         <v>5000000</v>
       </c>
     </row>
@@ -2733,7 +2725,7 @@
       <c r="B40" t="s">
         <v>89</v>
       </c>
-      <c r="C40" s="14">
+      <c r="C40" s="9">
         <v>3000000</v>
       </c>
     </row>
@@ -2741,7 +2733,7 @@
       <c r="B41" t="s">
         <v>73</v>
       </c>
-      <c r="C41" s="2">
+      <c r="C41" s="3">
         <f>C36+C37</f>
         <v>80000000</v>
       </c>
@@ -2750,7 +2742,7 @@
       <c r="B42" t="s">
         <v>78</v>
       </c>
-      <c r="C42" s="14">
+      <c r="C42" s="9">
         <v>50000000</v>
       </c>
     </row>
@@ -2758,7 +2750,7 @@
       <c r="B43" t="s">
         <v>90</v>
       </c>
-      <c r="C43" s="15">
+      <c r="C43" s="10">
         <v>0.1</v>
       </c>
     </row>
@@ -2766,7 +2758,7 @@
       <c r="B44" t="s">
         <v>93</v>
       </c>
-      <c r="C44" s="19">
+      <c r="C44" s="14">
         <f>'Sidekick Cap Table'!G21</f>
         <v>9740263</v>
       </c>
@@ -2775,7 +2767,7 @@
       <c r="B45" t="s">
         <v>94</v>
       </c>
-      <c r="C45" s="19">
+      <c r="C45" s="14">
         <f>'SAFE Investments'!C24</f>
         <v>9825000</v>
       </c>
@@ -2784,7 +2776,7 @@
       <c r="B46" t="s">
         <v>91</v>
       </c>
-      <c r="C46" s="19">
+      <c r="C46" s="14">
         <f>'Sidekick Cap Table'!G20</f>
         <v>65105</v>
       </c>
@@ -2793,7 +2785,7 @@
       <c r="B47" t="s">
         <v>95</v>
       </c>
-      <c r="C47" s="18">
+      <c r="C47" s="13">
         <f>C42/C44</f>
         <v>5.1333316153783528</v>
       </c>
@@ -2802,7 +2794,7 @@
       <c r="B48" t="s">
         <v>96</v>
       </c>
-      <c r="C48" s="2">
+      <c r="C48" s="3">
         <f>C45/C47</f>
         <v>1913961.6794999999</v>
       </c>
@@ -2811,7 +2803,7 @@
       <c r="B49" t="s">
         <v>97</v>
       </c>
-      <c r="C49" s="2">
+      <c r="C49" s="3">
         <f>(C44+C48-C46)/(1-C43-C37/C41)</f>
         <v>17829414.891538464</v>
       </c>
@@ -2820,7 +2812,7 @@
       <c r="B50" t="s">
         <v>98</v>
       </c>
-      <c r="C50" s="18">
+      <c r="C50" s="13">
         <f>C41/C49</f>
         <v>4.48696721045886</v>
       </c>
@@ -2829,7 +2821,7 @@
       <c r="B51" t="s">
         <v>99</v>
       </c>
-      <c r="C51" s="2">
+      <c r="C51" s="3">
         <f>C37/C50</f>
         <v>4457353.7228846159</v>
       </c>
@@ -2838,18 +2830,9 @@
       <c r="B52" t="s">
         <v>92</v>
       </c>
-      <c r="C52" s="2">
+      <c r="C52" s="3">
         <f>C43*C49-C46</f>
         <v>1717836.4891538464</v>
-      </c>
-    </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B53" t="s">
-        <v>100</v>
-      </c>
-      <c r="C53" s="2">
-        <f>C38+C39+C40-C37</f>
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2858,12 +2841,12 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AF22BCC-A6D7-6749-9B46-9E072129FD10}">
-  <dimension ref="A1:R51"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60CD3F6A-DC0D-414A-8C03-BA348FCB8396}">
+  <dimension ref="A1:R53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.83203125" customWidth="1"/>
-    <col min="2" max="2" width="51.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
@@ -2877,13 +2860,13 @@
     <col min="14" max="14" width="3.83203125" customWidth="1"/>
     <col min="15" max="15" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="3.83203125" customWidth="1"/>
-    <col min="17" max="17" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="8.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B1" s="6" t="s">
-        <v>114</v>
+      <c r="B1" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
@@ -2963,44 +2946,44 @@
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" s="12"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12" t="s">
+      <c r="A5" s="18"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12" t="s">
+      <c r="F5" s="18"/>
+      <c r="G5" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="H5" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12" t="s">
+      <c r="I5" s="18"/>
+      <c r="J5" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12" t="s">
+      <c r="K5" s="18"/>
+      <c r="L5" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="M5" s="12" t="s">
+      <c r="M5" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="N5" s="12"/>
-      <c r="O5" s="12" t="s">
+      <c r="N5" s="18"/>
+      <c r="O5" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="P5" s="12"/>
-      <c r="Q5" s="12" t="s">
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="R5" s="12" t="s">
+      <c r="R5" s="18" t="s">
         <v>64</v>
       </c>
     </row>
@@ -3013,24 +2996,24 @@
       <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="14">
         <f>'Series A'!C7</f>
         <v>3600000</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="Q7" s="2">
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="Q7" s="3">
         <f>C7</f>
         <v>3600000</v>
       </c>
-      <c r="R7" s="3">
-        <f>Q7/$C$47</f>
+      <c r="R7" s="4">
+        <f>Q7/$C$49</f>
         <v>0.15648298146475273</v>
       </c>
     </row>
@@ -3038,24 +3021,24 @@
       <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="14">
         <f>'Series A'!C8</f>
         <v>3600000</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="Q8" s="2">
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="Q8" s="3">
         <f>C8</f>
         <v>3600000</v>
       </c>
-      <c r="R8" s="3">
-        <f>Q8/$C$47</f>
+      <c r="R8" s="4">
+        <f>Q8/$C$49</f>
         <v>0.15648298146475273</v>
       </c>
     </row>
@@ -3063,24 +3046,24 @@
       <c r="B9" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="14">
         <f>'Series A'!C9</f>
         <v>592500</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="Q9" s="2">
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="Q9" s="3">
         <f>C9</f>
         <v>592500</v>
       </c>
-      <c r="R9" s="3">
-        <f>Q9/$C$47</f>
+      <c r="R9" s="4">
+        <f>Q9/$C$49</f>
         <v>2.5754490699407218E-2</v>
       </c>
     </row>
@@ -3088,24 +3071,24 @@
       <c r="B10" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="19">
+      <c r="C10" s="14">
         <f>'Series A'!C10</f>
         <v>592500</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="Q10" s="2">
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="Q10" s="3">
         <f>C10</f>
         <v>592500</v>
       </c>
-      <c r="R10" s="3">
-        <f>Q10/$C$47</f>
+      <c r="R10" s="4">
+        <f>Q10/$C$49</f>
         <v>2.5754490699407218E-2</v>
       </c>
     </row>
@@ -3113,24 +3096,24 @@
       <c r="B11" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="14">
         <f>'Series A'!C11</f>
         <v>222187</v>
       </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="Q11" s="2">
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="Q11" s="3">
         <f>C11</f>
         <v>222187</v>
       </c>
-      <c r="R11" s="3">
-        <f>Q11/$C$47</f>
+      <c r="R11" s="4">
+        <f>Q11/$C$49</f>
         <v>9.6579122785302816E-3</v>
       </c>
     </row>
@@ -3138,24 +3121,24 @@
       <c r="B12" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="14">
         <f>'Series A'!C12</f>
         <v>285000</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-      <c r="O12" s="2"/>
-      <c r="Q12" s="2">
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="O12" s="3"/>
+      <c r="Q12" s="3">
         <f>C12</f>
         <v>285000</v>
       </c>
-      <c r="R12" s="3">
-        <f>Q12/$C$47</f>
+      <c r="R12" s="4">
+        <f>Q12/$C$49</f>
         <v>1.2388236032626256E-2</v>
       </c>
     </row>
@@ -3163,24 +3146,24 @@
       <c r="B13" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="14">
         <f>'Series A'!C13</f>
         <v>285000</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="Q13" s="2">
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="O13" s="3"/>
+      <c r="Q13" s="3">
         <f>C13</f>
         <v>285000</v>
       </c>
-      <c r="R13" s="3">
-        <f>Q13/$C$47</f>
+      <c r="R13" s="4">
+        <f>Q13/$C$49</f>
         <v>1.2388236032626256E-2</v>
       </c>
     </row>
@@ -3188,24 +3171,24 @@
       <c r="B14" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="14">
         <f>'Series A'!C14</f>
         <v>112400</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="Q14" s="2">
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="O14" s="3"/>
+      <c r="Q14" s="3">
         <f>C14</f>
         <v>112400</v>
       </c>
-      <c r="R14" s="3">
-        <f>Q14/$C$47</f>
+      <c r="R14" s="4">
+        <f>Q14/$C$49</f>
         <v>4.8857464212883903E-3</v>
       </c>
     </row>
@@ -3213,24 +3196,24 @@
       <c r="B15" t="s">
         <v>85</v>
       </c>
-      <c r="C15" s="19">
+      <c r="C15" s="14">
         <f>'Series A'!C15</f>
         <v>385571</v>
       </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="Q15" s="2">
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="O15" s="3"/>
+      <c r="Q15" s="3">
         <f>C15</f>
         <v>385571</v>
       </c>
-      <c r="R15" s="3">
-        <f>Q15/$C$47</f>
+      <c r="R15" s="4">
+        <f>Q15/$C$49</f>
         <v>1.675980545731838E-2</v>
       </c>
     </row>
@@ -3238,30 +3221,30 @@
       <c r="B16" t="s">
         <v>86</v>
       </c>
-      <c r="C16" s="19">
+      <c r="C16" s="14">
         <f>'Series A'!C16</f>
         <v>65105</v>
       </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="J16" s="19">
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="J16" s="14">
         <f>'Series A'!J16</f>
         <v>1717836.4891538464</v>
       </c>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="O16" s="2">
-        <f>$C$48</f>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3"/>
+      <c r="O16" s="3">
+        <f>$C$50</f>
         <v>1610398.764397023</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16" s="3">
         <f>C16+J16+O16</f>
         <v>3393340.2535508694</v>
       </c>
-      <c r="R16" s="3">
-        <f>Q16/$C$47</f>
+      <c r="R16" s="4">
+        <f>Q16/$C$49</f>
         <v>0.14749999999999999</v>
       </c>
     </row>
@@ -3269,104 +3252,104 @@
       <c r="B17" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="5">
         <f>SUM(C7:C16)</f>
         <v>9740263</v>
       </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="4">
+      <c r="J17" s="5">
         <f>SUM(J7:J16)</f>
         <v>1717836.4891538464</v>
       </c>
       <c r="K17" s="1"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
       <c r="N17" s="1"/>
-      <c r="O17" s="4">
+      <c r="O17" s="5">
         <f>SUM(O7:O16)</f>
         <v>1610398.764397023</v>
       </c>
       <c r="P17" s="1"/>
-      <c r="Q17" s="4">
+      <c r="Q17" s="5">
         <f>SUM(Q7:Q16)</f>
         <v>13068498.253550868</v>
       </c>
-      <c r="R17" s="5">
-        <f>Q17/$C$47</f>
+      <c r="R17" s="6">
+        <f>Q17/$C$49</f>
         <v>0.56805488055070941</v>
       </c>
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-      <c r="O18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3"/>
+      <c r="O18" s="3"/>
+      <c r="Q18" s="3"/>
+      <c r="R18" s="4"/>
     </row>
     <row r="19" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
-      <c r="O19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
+      <c r="O19" s="3"/>
+      <c r="Q19" s="3"/>
+      <c r="R19" s="4"/>
     </row>
     <row r="20" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>87</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="19">
+      <c r="C20" s="3"/>
+      <c r="D20" s="14">
         <f>'Series A'!D20</f>
         <v>8000000</v>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="14">
         <f>'Series A'!E20</f>
         <v>1558442.08</v>
       </c>
-      <c r="G20" s="19">
+      <c r="G20" s="14">
         <f>'Series A'!G20</f>
         <v>5000000</v>
       </c>
-      <c r="H20" s="19">
+      <c r="H20" s="14">
         <f>'Series A'!H20</f>
         <v>1114338.430721154</v>
       </c>
-      <c r="J20" s="2"/>
-      <c r="L20" s="2">
-        <f>$C$50</f>
+      <c r="J20" s="3"/>
+      <c r="L20" s="3">
+        <f>$C$52</f>
         <v>3750000</v>
       </c>
-      <c r="M20" s="2">
-        <f>L20/$C$44</f>
+      <c r="M20" s="3">
+        <f>L20/$C$46</f>
         <v>445735.3722884616</v>
       </c>
-      <c r="O20" s="2"/>
-      <c r="Q20" s="2">
+      <c r="O20" s="3"/>
+      <c r="Q20" s="3">
         <f>E20+H20+M20</f>
         <v>3118515.8830096158</v>
       </c>
-      <c r="R20" s="3">
-        <f>Q20/$C$47</f>
+      <c r="R20" s="4">
+        <f>Q20/$C$49</f>
         <v>0.13555407308848075</v>
       </c>
     </row>
@@ -3374,27 +3357,27 @@
       <c r="B21" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="19">
+      <c r="C21" s="3"/>
+      <c r="D21" s="14">
         <f>'Series A'!D21</f>
         <v>250000</v>
       </c>
-      <c r="E21" s="19">
+      <c r="E21" s="14">
         <f>'Series A'!E21</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
-      <c r="O21" s="2"/>
-      <c r="Q21" s="2">
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="O21" s="3"/>
+      <c r="Q21" s="3">
         <f>E21</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="R21" s="3">
-        <f>Q21/$C$47</f>
+      <c r="R21" s="4">
+        <f>Q21/$C$49</f>
         <v>2.1169241590150234E-3</v>
       </c>
     </row>
@@ -3402,27 +3385,27 @@
       <c r="B22" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="19">
+      <c r="C22" s="3"/>
+      <c r="D22" s="14">
         <f>'Series A'!D22</f>
         <v>300000</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="14">
         <f>'Series A'!E22</f>
         <v>58441.578000000001</v>
       </c>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-      <c r="O22" s="2"/>
-      <c r="Q22" s="2">
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
+      <c r="O22" s="3"/>
+      <c r="Q22" s="3">
         <f>E22</f>
         <v>58441.578000000001</v>
       </c>
-      <c r="R22" s="3">
-        <f>Q22/$C$47</f>
+      <c r="R22" s="4">
+        <f>Q22/$C$49</f>
         <v>2.5403089908180281E-3</v>
       </c>
     </row>
@@ -3430,27 +3413,27 @@
       <c r="B23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="19">
+      <c r="C23" s="3"/>
+      <c r="D23" s="14">
         <f>'Series A'!D23</f>
         <v>250000</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="14">
         <f>'Series A'!E23</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-      <c r="O23" s="2"/>
-      <c r="Q23" s="2">
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="Q23" s="3">
         <f>E23</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="R23" s="3">
-        <f>Q23/$C$47</f>
+      <c r="R23" s="4">
+        <f>Q23/$C$49</f>
         <v>2.1169241590150234E-3</v>
       </c>
     </row>
@@ -3458,27 +3441,27 @@
       <c r="B24" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="19">
+      <c r="C24" s="3"/>
+      <c r="D24" s="14">
         <f>'Series A'!D24</f>
         <v>212500</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="14">
         <f>'Series A'!E24</f>
         <v>41396.117749999998</v>
       </c>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="Q24" s="2">
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="O24" s="3"/>
+      <c r="Q24" s="3">
         <f>E24</f>
         <v>41396.117749999998</v>
       </c>
-      <c r="R24" s="3">
-        <f>Q24/$C$47</f>
+      <c r="R24" s="4">
+        <f>Q24/$C$49</f>
         <v>1.7993855351627697E-3</v>
       </c>
     </row>
@@ -3486,27 +3469,27 @@
       <c r="B25" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="19">
+      <c r="C25" s="3"/>
+      <c r="D25" s="14">
         <f>'Series A'!D25</f>
         <v>250000</v>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="14">
         <f>'Series A'!E25</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="Q25" s="2">
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="Q25" s="3">
         <f>E25</f>
         <v>48701.315000000002</v>
       </c>
-      <c r="R25" s="3">
-        <f>Q25/$C$47</f>
+      <c r="R25" s="4">
+        <f>Q25/$C$49</f>
         <v>2.1169241590150234E-3</v>
       </c>
     </row>
@@ -3514,27 +3497,27 @@
       <c r="B26" t="s">
         <v>88</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="19">
+      <c r="C26" s="3"/>
+      <c r="D26" s="14">
         <f>'Series A'!D26</f>
         <v>562500</v>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="14">
         <f>'Series A'!E26</f>
         <v>109577.95875000001</v>
       </c>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-      <c r="O26" s="2"/>
-      <c r="Q26" s="2">
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="O26" s="3"/>
+      <c r="Q26" s="3">
         <f>E26</f>
         <v>109577.95875000001</v>
       </c>
-      <c r="R26" s="3">
-        <f>Q26/$C$47</f>
+      <c r="R26" s="4">
+        <f>Q26/$C$49</f>
         <v>4.7630793577838025E-3</v>
       </c>
     </row>
@@ -3542,33 +3525,33 @@
       <c r="B27" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="G27" s="19">
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="G27" s="14">
         <f>'Series A'!G27</f>
         <v>12000000</v>
       </c>
-      <c r="H27" s="19">
+      <c r="H27" s="14">
         <f>'Series A'!H27</f>
         <v>2674412.2337307697</v>
       </c>
-      <c r="J27" s="2"/>
-      <c r="L27" s="2">
-        <f>$C$49</f>
+      <c r="J27" s="3"/>
+      <c r="L27" s="3">
+        <f>$C$51</f>
         <v>9000000</v>
       </c>
-      <c r="M27" s="2">
-        <f>L27/$C$44</f>
+      <c r="M27" s="3">
+        <f>L27/$C$46</f>
         <v>1069764.8934923077</v>
       </c>
-      <c r="O27" s="2"/>
-      <c r="Q27" s="2">
+      <c r="O27" s="3"/>
+      <c r="Q27" s="3">
         <f>H27+M27</f>
         <v>3744177.1272230772</v>
       </c>
-      <c r="R27" s="3">
-        <f>Q27/$C$47</f>
+      <c r="R27" s="4">
+        <f>Q27/$C$49</f>
         <v>0.16274999999999998</v>
       </c>
     </row>
@@ -3576,146 +3559,146 @@
       <c r="B28" t="s">
         <v>69</v>
       </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="G28" s="19">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="G28" s="14">
         <f>'Series A'!G28</f>
         <v>3000000</v>
       </c>
-      <c r="H28" s="19">
+      <c r="H28" s="14">
         <f>'Series A'!H28</f>
         <v>668603.05843269243</v>
       </c>
-      <c r="J28" s="2"/>
-      <c r="L28" s="2">
-        <f>$C$51</f>
+      <c r="J28" s="3"/>
+      <c r="L28" s="3">
+        <f>$C$53</f>
         <v>2250000</v>
       </c>
-      <c r="M28" s="2">
-        <f>L28/$C$44</f>
+      <c r="M28" s="3">
+        <f>L28/$C$46</f>
         <v>267441.22337307694</v>
       </c>
-      <c r="O28" s="2"/>
-      <c r="Q28" s="2">
+      <c r="O28" s="3"/>
+      <c r="Q28" s="3">
         <f>H28+M28</f>
         <v>936044.28180576931</v>
       </c>
-      <c r="R28" s="3">
-        <f>Q28/$C$47</f>
+      <c r="R28" s="4">
+        <f>Q28/$C$49</f>
         <v>4.0687499999999995E-2</v>
       </c>
     </row>
     <row r="29" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B29" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="L29" s="2">
-        <f>$C$38</f>
+        <v>112</v>
+      </c>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="L29" s="3">
+        <f>$C$40</f>
         <v>15000000</v>
       </c>
-      <c r="M29" s="2">
-        <f>L29/$C$44</f>
+      <c r="M29" s="3">
+        <f>L29/$C$46</f>
         <v>1782941.4891538464</v>
       </c>
-      <c r="O29" s="2"/>
-      <c r="Q29" s="2">
+      <c r="O29" s="3"/>
+      <c r="Q29" s="3">
         <f>M29</f>
         <v>1782941.4891538464</v>
       </c>
-      <c r="R29" s="3">
-        <f>Q29/$C$47</f>
+      <c r="R29" s="4">
+        <f>Q29/$C$49</f>
         <v>7.7499999999999986E-2</v>
       </c>
     </row>
     <row r="30" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-      <c r="O30" s="2"/>
-      <c r="Q30" s="2"/>
-      <c r="R30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="O30" s="3"/>
+      <c r="Q30" s="3"/>
+      <c r="R30" s="4"/>
     </row>
     <row r="31" spans="2:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="11">
         <f>SUM(C7:C16)</f>
         <v>9740263</v>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="11">
         <f>SUM(D20:D26)</f>
         <v>9825000</v>
       </c>
-      <c r="E31" s="16">
+      <c r="E31" s="11">
         <f>SUM(E20:E26)</f>
         <v>1913961.6794999999</v>
       </c>
-      <c r="F31" s="13"/>
-      <c r="G31" s="16">
+      <c r="F31" s="8"/>
+      <c r="G31" s="11">
         <f>SUM(G20:G28)</f>
         <v>20000000</v>
       </c>
-      <c r="H31" s="16">
+      <c r="H31" s="11">
         <f>SUM(H20:H28)</f>
         <v>4457353.7228846159</v>
       </c>
-      <c r="I31" s="13"/>
-      <c r="J31" s="16">
+      <c r="I31" s="8"/>
+      <c r="J31" s="11">
         <f>J16</f>
         <v>1717836.4891538464</v>
       </c>
-      <c r="K31" s="13"/>
-      <c r="L31" s="16">
+      <c r="K31" s="8"/>
+      <c r="L31" s="11">
         <f>SUM(L20:L29)</f>
         <v>30000000</v>
       </c>
-      <c r="M31" s="16">
+      <c r="M31" s="11">
         <f>SUM(M20:M29)</f>
         <v>3565882.9783076923</v>
       </c>
-      <c r="N31" s="13"/>
-      <c r="O31" s="16">
+      <c r="N31" s="8"/>
+      <c r="O31" s="11">
         <f>O16</f>
         <v>1610398.764397023</v>
       </c>
-      <c r="P31" s="13"/>
-      <c r="Q31" s="16">
+      <c r="P31" s="8"/>
+      <c r="Q31" s="11">
         <f>C31+E31+H31+J31+M31+O31</f>
         <v>23005696.634243179</v>
       </c>
-      <c r="R31" s="17">
-        <f>Q31/$C$47</f>
+      <c r="R31" s="12">
+        <f>Q31/$C$49</f>
         <v>0.99999999999999989</v>
       </c>
     </row>
     <row r="32" spans="2:18" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B33" s="20" t="s">
+      <c r="B33" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="E33" s="21">
+      <c r="E33" s="16">
         <f>'Series A'!E32</f>
         <v>5.1333316153783528</v>
       </c>
-      <c r="H33" s="21">
+      <c r="H33" s="16">
         <f>'Series A'!H32</f>
         <v>4.48696721045886</v>
       </c>
-      <c r="M33" s="18">
-        <f>$C$44</f>
+      <c r="M33" s="13">
+        <f>$C$46</f>
         <v>8.4130635196103629</v>
       </c>
     </row>
@@ -3723,161 +3706,169 @@
       <c r="B34" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E34" s="19">
+      <c r="E34" s="14">
         <f>'Series A'!E33</f>
         <v>50000000</v>
       </c>
-      <c r="H34" s="19">
+      <c r="H34" s="14">
         <f>'Series A'!H33</f>
         <v>60000000</v>
       </c>
-      <c r="M34" s="2">
-        <f>$C$36</f>
+      <c r="M34" s="3">
+        <f>$C$38</f>
         <v>150000000</v>
       </c>
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E35" s="14">
+        <f>'Series A'!E34</f>
+        <v>50000000</v>
+      </c>
+      <c r="H35" s="14">
+        <f>'Series A'!H34</f>
+        <v>80000000</v>
+      </c>
+      <c r="M35" s="3">
+        <f>$C$43</f>
+        <v>180000000</v>
+      </c>
+    </row>
+    <row r="37" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B37" s="1" t="s">
         <v>81</v>
-      </c>
-    </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B36" t="s">
-        <v>72</v>
-      </c>
-      <c r="C36" s="14">
-        <v>150000000</v>
-      </c>
-    </row>
-    <row r="37" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B37" t="s">
-        <v>75</v>
-      </c>
-      <c r="C37" s="14">
-        <v>30000000</v>
       </c>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>101</v>
-      </c>
-      <c r="C38" s="14">
-        <v>15000000</v>
+        <v>72</v>
+      </c>
+      <c r="C38" s="9">
+        <v>150000000</v>
       </c>
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>102</v>
-      </c>
-      <c r="C39" s="2">
-        <f>C37-C38</f>
-        <v>15000000</v>
+        <v>75</v>
+      </c>
+      <c r="C39" s="9">
+        <v>30000000</v>
       </c>
     </row>
     <row r="40" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>103</v>
-      </c>
-      <c r="C40" s="15">
-        <v>7.0000000000000007E-2</v>
+        <v>100</v>
+      </c>
+      <c r="C40" s="9">
+        <v>15000000</v>
       </c>
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
-        <v>73</v>
-      </c>
-      <c r="C41" s="2">
-        <f>C36+C37</f>
-        <v>180000000</v>
+        <v>101</v>
+      </c>
+      <c r="C41" s="3">
+        <f>C39-C40</f>
+        <v>15000000</v>
       </c>
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
-        <v>104</v>
-      </c>
-      <c r="C42" s="19">
+        <v>102</v>
+      </c>
+      <c r="C42" s="10">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="3">
+        <f>C38+C39</f>
+        <v>180000000</v>
+      </c>
+    </row>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
+        <v>103</v>
+      </c>
+      <c r="C44" s="14">
         <f>'Series A'!C49</f>
         <v>17829414.891538464</v>
       </c>
     </row>
-    <row r="43" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B43" t="s">
-        <v>105</v>
-      </c>
-      <c r="C43" s="19">
-        <f>'Series A'!L16</f>
-        <v>1782941.4891538464</v>
-      </c>
-    </row>
-    <row r="44" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B44" t="s">
-        <v>106</v>
-      </c>
-      <c r="C44" s="18">
-        <f>C36/C42</f>
-        <v>8.4130635196103629</v>
-      </c>
-    </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B45" t="s">
-        <v>107</v>
-      </c>
-      <c r="C45" s="2">
-        <f>C37/C44</f>
-        <v>3565882.9783076928</v>
-      </c>
-    </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>108</v>
-      </c>
-      <c r="C46" s="2">
-        <f>C42+C45</f>
-        <v>21395297.869846158</v>
+        <v>104</v>
+      </c>
+      <c r="C46" s="13">
+        <f>C38/C44</f>
+        <v>8.4130635196103629</v>
       </c>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
-        <v>109</v>
-      </c>
-      <c r="C47" s="2">
-        <f>C46/(1-C40)</f>
-        <v>23005696.634243183</v>
+        <v>105</v>
+      </c>
+      <c r="C47" s="3">
+        <f>C39/C46</f>
+        <v>3565882.9783076928</v>
       </c>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
-        <v>110</v>
-      </c>
-      <c r="C48" s="2">
-        <f>C40*C47</f>
-        <v>1610398.764397023</v>
+        <v>106</v>
+      </c>
+      <c r="C48" s="3">
+        <f>C44+C47</f>
+        <v>21395297.869846158</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
-        <v>111</v>
-      </c>
-      <c r="C49" s="19">
-        <f>C39*'Series A'!C38/'Series A'!C37</f>
-        <v>9000000</v>
+        <v>107</v>
+      </c>
+      <c r="C49" s="3">
+        <f>C48/(1-C42)</f>
+        <v>23005696.634243183</v>
       </c>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
-        <v>112</v>
-      </c>
-      <c r="C50" s="19">
-        <f>C39*'Series A'!C39/'Series A'!C37</f>
-        <v>3750000</v>
+        <v>108</v>
+      </c>
+      <c r="C50" s="3">
+        <f>C42*C49</f>
+        <v>1610398.764397023</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
+        <v>109</v>
+      </c>
+      <c r="C51" s="14">
+        <f>C41*'Series A'!C38/'Series A'!C37</f>
+        <v>9000000</v>
+      </c>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B52" t="s">
+        <v>110</v>
+      </c>
+      <c r="C52" s="14">
+        <f>C41*'Series A'!C39/'Series A'!C37</f>
+        <v>3750000</v>
+      </c>
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B53" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="19">
-        <f>C39*'Series A'!C40/'Series A'!C37</f>
+      <c r="C53" s="14">
+        <f>C41*'Series A'!C40/'Series A'!C37</f>
         <v>2250000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Checkpoint: Series A sheet - corrected with post-money SAFE mechanics and individual holders
</commit_message>
<xml_diff>
--- a/runs/resume/models/model.xlsx
+++ b/runs/resume/models/model.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3A0C140-B4E9-BD43-BE99-76D775A2F664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA05ADCB-0193-A34E-ABDF-5F5B6D501518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__temp__" sheetId="72" r:id="rId1"/>
     <sheet name="Sidekick Cap Table" sheetId="73" r:id="rId2"/>
     <sheet name="SAFE Investments" sheetId="74" r:id="rId3"/>
+    <sheet name="Series A" sheetId="77" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="91">
   <si>
     <t>Total</t>
   </si>
@@ -193,17 +194,136 @@
     <t>Mark Lotke</t>
   </si>
   <si>
+    <t>SIDEKICK (THINK MORE SECURITY, INC.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Common </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option </t>
+  </si>
+  <si>
+    <t>Series A</t>
+  </si>
+  <si>
+    <t>Total Capitalization</t>
+  </si>
+  <si>
+    <t># of</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Preferred</t>
+  </si>
+  <si>
+    <t>Pool +</t>
+  </si>
+  <si>
+    <t>Total FD</t>
+  </si>
+  <si>
+    <t>Shares</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Invested</t>
+  </si>
+  <si>
+    <t>SAFE Shares</t>
+  </si>
+  <si>
+    <t>FD</t>
+  </si>
+  <si>
+    <t>Common Stock and Options:</t>
+  </si>
+  <si>
+    <t>Total Common</t>
+  </si>
+  <si>
+    <t>Preferred Rounds</t>
+  </si>
+  <si>
+    <t>1011 Ventures</t>
+  </si>
+  <si>
+    <t>Other Series A Investors</t>
+  </si>
+  <si>
+    <t>Totals</t>
+  </si>
+  <si>
+    <t>Price per Share</t>
+  </si>
+  <si>
+    <t>Pre-Money Valuation</t>
+  </si>
+  <si>
+    <t>Post-Money Valuation</t>
+  </si>
+  <si>
+    <t>Series A Assumptions:</t>
+  </si>
+  <si>
+    <t>Total Raised</t>
+  </si>
+  <si>
+    <t>Option Pool Target (% post-money)</t>
+  </si>
+  <si>
+    <t>Other Series A</t>
+  </si>
+  <si>
+    <t>Small Common Holders</t>
+  </si>
+  <si>
+    <t>Pre-A</t>
+  </si>
+  <si>
+    <t>Post-A</t>
+  </si>
+  <si>
+    <t>Accomplice Series A</t>
+  </si>
+  <si>
     <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
+  </si>
+  <si>
+    <t>SIDEKICK &amp; 1011 VENTURES / ACCOMPLICE SERIES A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% </t>
+  </si>
+  <si>
+    <t>% Ownership (Series A)</t>
+  </si>
+  <si>
+    <t>SAFE Post-Money Val Cap</t>
+  </si>
+  <si>
+    <t>1011 Contribution</t>
+  </si>
+  <si>
+    <t>Elizabeth A. Donaghey Irrevocable Trust</t>
+  </si>
+  <si>
+    <t>Small SAFE Investors</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="_-[$$-409]* #,##0_-;_-[$$-409]* \(#,##0\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
+    <numFmt numFmtId="169" formatCode="0.0%_);\(0.0%\);0.0%_);@_)"/>
+    <numFmt numFmtId="171" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\);&quot;$&quot;#,##0_);@_)"/>
+    <numFmt numFmtId="175" formatCode="_-[$$-409]* #,##0.0000_-;_-[$$-409]* \(#,##0.0000\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -339,6 +459,31 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -351,8 +496,15 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -532,8 +684,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -648,6 +806,145 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -693,8 +990,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -707,22 +1005,107 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="20" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="171" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="37" fontId="18" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="18" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="169" fontId="18" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="18" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="18" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="18" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="37" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1144,495 +1527,495 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
+      <c r="A1" s="5"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="6" t="s">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="4"/>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="4"/>
-      <c r="B4" s="5" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="12">
         <v>3600000</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7">
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="13">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="4"/>
-      <c r="B5" s="5" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="12">
         <v>3600000</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7">
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="13">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="4"/>
-      <c r="B6" s="5" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="12">
         <v>222187</v>
       </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7">
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="13">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="4"/>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="12">
         <v>592500</v>
       </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7">
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="13">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="12">
         <v>592500</v>
       </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7">
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="13">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="4"/>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="5"/>
+      <c r="B9" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="12">
         <v>13500</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="12">
         <v>98900</v>
       </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7">
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="13">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="4"/>
-      <c r="B10" s="5" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="12">
         <v>9000</v>
       </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7">
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="13">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="4"/>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7">
+      <c r="C11" s="12"/>
+      <c r="D11" s="12">
         <v>95000</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7">
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="13">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="5" t="s">
+      <c r="A12" s="5"/>
+      <c r="B12" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7">
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12">
         <v>25000</v>
       </c>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7">
+      <c r="F12" s="12"/>
+      <c r="G12" s="12">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="13">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="4"/>
-      <c r="B13" s="5" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7">
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12">
         <v>41562</v>
       </c>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7">
+      <c r="F13" s="12"/>
+      <c r="G13" s="12">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="13">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="4"/>
-      <c r="B14" s="5" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7">
+      <c r="C14" s="12"/>
+      <c r="D14" s="12">
         <v>285000</v>
       </c>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7">
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="13">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="4"/>
-      <c r="B15" s="5" t="s">
+      <c r="A15" s="5"/>
+      <c r="B15" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7">
+      <c r="C15" s="12"/>
+      <c r="D15" s="12">
         <v>50000</v>
       </c>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7">
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="8">
+      <c r="H15" s="13">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="4"/>
-      <c r="B16" s="5" t="s">
+      <c r="A16" s="5"/>
+      <c r="B16" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7">
+      <c r="C16" s="12"/>
+      <c r="D16" s="12">
         <v>285000</v>
       </c>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7">
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="13">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="4"/>
-      <c r="B17" s="5" t="s">
+      <c r="A17" s="5"/>
+      <c r="B17" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7">
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12">
         <v>96186</v>
       </c>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7">
+      <c r="F17" s="12"/>
+      <c r="G17" s="12">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="8">
+      <c r="H17" s="13">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
-      <c r="B18" s="5" t="s">
+      <c r="A18" s="5"/>
+      <c r="B18" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7">
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12">
         <v>48095</v>
       </c>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7">
+      <c r="F18" s="12"/>
+      <c r="G18" s="12">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="13">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="4"/>
-      <c r="B19" s="5" t="s">
+      <c r="A19" s="5"/>
+      <c r="B19" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7">
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12">
         <v>12395</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="12">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="13">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" s="4"/>
-      <c r="B20" s="5" t="s">
+      <c r="A20" s="5"/>
+      <c r="B20" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7">
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12">
         <v>8333</v>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="12">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="8">
+      <c r="H20" s="13">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
     </row>
     <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="4"/>
-      <c r="B21" s="5" t="s">
+      <c r="A21" s="5"/>
+      <c r="B21" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7">
+      <c r="C21" s="12"/>
+      <c r="D21" s="12">
         <v>65105</v>
       </c>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7">
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H21" s="13">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
     </row>
     <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
     </row>
     <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="4"/>
-      <c r="B23" s="6" t="s">
+      <c r="A23" s="5"/>
+      <c r="B23" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="12">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="7">
+      <c r="D23" s="12">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="7">
+      <c r="E23" s="12">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="7">
+      <c r="F23" s="12">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="7">
+      <c r="G23" s="12">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="2"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1653,341 +2036,1232 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
+      <c r="A1" s="5"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="4"/>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="6" t="s">
+      <c r="D3" s="5"/>
+      <c r="E3" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="4"/>
+      <c r="F3" s="5"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="4"/>
-      <c r="B4" s="5" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="14">
         <v>25000</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="5" t="s">
+      <c r="D4" s="5"/>
+      <c r="E4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="4"/>
+      <c r="F4" s="5"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="4"/>
-      <c r="B5" s="5" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="14">
         <v>25000</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="4"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="5"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="4"/>
-      <c r="B6" s="5" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="14">
         <v>137170.75</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="4"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="5"/>
     </row>
     <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="4"/>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="14">
         <v>3846829.25</v>
       </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="4"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="5"/>
     </row>
     <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="14">
         <v>16566</v>
       </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="4"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="4"/>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="5"/>
+      <c r="B9" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="14">
         <v>250000</v>
       </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="4"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="5"/>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="4"/>
-      <c r="B10" s="5" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="14">
         <v>100000</v>
       </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="4"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="5"/>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="4"/>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="14">
         <v>300000</v>
       </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="5" t="s">
+      <c r="D11" s="5"/>
+      <c r="E11" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="4"/>
+      <c r="F11" s="5"/>
     </row>
     <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="5" t="s">
+      <c r="A12" s="5"/>
+      <c r="B12" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="14">
         <v>37500</v>
       </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="5" t="s">
+      <c r="D12" s="5"/>
+      <c r="E12" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="4"/>
+      <c r="F12" s="5"/>
     </row>
     <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="4"/>
-      <c r="B13" s="5" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="14">
         <v>250000</v>
       </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="4"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="5"/>
     </row>
     <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="4"/>
-      <c r="B14" s="5" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="14">
         <v>100000</v>
       </c>
-      <c r="D14" s="4"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="4"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="5"/>
     </row>
     <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="4"/>
-      <c r="B15" s="5" t="s">
+      <c r="A15" s="5"/>
+      <c r="B15" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="14">
         <v>41164</v>
       </c>
-      <c r="D15" s="4"/>
-      <c r="E15" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F15" s="4"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F15" s="5"/>
     </row>
     <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="4"/>
-      <c r="B16" s="5" t="s">
+      <c r="A16" s="5"/>
+      <c r="B16" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="14">
         <v>2328778</v>
       </c>
-      <c r="D16" s="4"/>
-      <c r="E16" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F16" s="4"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="5"/>
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="4"/>
-      <c r="B17" s="5" t="s">
+      <c r="A17" s="5"/>
+      <c r="B17" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="14">
         <v>1506000</v>
       </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="5" t="s">
+      <c r="D17" s="5"/>
+      <c r="E17" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="4"/>
+      <c r="F17" s="5"/>
     </row>
     <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
-      <c r="B18" s="5" t="s">
+      <c r="A18" s="5"/>
+      <c r="B18" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="14">
         <v>50000</v>
       </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="4"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="5"/>
     </row>
     <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="4"/>
-      <c r="B19" s="5" t="s">
+      <c r="A19" s="5"/>
+      <c r="B19" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="14">
         <v>212500</v>
       </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="5" t="s">
+      <c r="D19" s="5"/>
+      <c r="E19" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="4"/>
+      <c r="F19" s="5"/>
     </row>
     <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="4"/>
-      <c r="B20" s="5" t="s">
+      <c r="A20" s="5"/>
+      <c r="B20" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="14">
         <v>25000</v>
       </c>
-      <c r="D20" s="4"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="4"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="5"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="4"/>
-      <c r="B21" s="5" t="s">
+      <c r="A21" s="5"/>
+      <c r="B21" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="14">
         <v>61746</v>
       </c>
-      <c r="D21" s="4"/>
-      <c r="E21" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F21" s="4"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F21" s="5"/>
     </row>
     <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="4"/>
-      <c r="B22" s="5" t="s">
+      <c r="A22" s="5"/>
+      <c r="B22" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="9">
+      <c r="C22" s="14">
         <v>100000</v>
       </c>
-      <c r="D22" s="4"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="4"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="5"/>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="4"/>
-      <c r="B23" s="5" t="s">
+      <c r="A23" s="5"/>
+      <c r="B23" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="14">
         <v>100000</v>
       </c>
-      <c r="D23" s="4"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="4"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="5"/>
     </row>
     <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="4"/>
-      <c r="B24" s="5" t="s">
+      <c r="A24" s="5"/>
+      <c r="B24" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="14">
         <v>61746</v>
       </c>
-      <c r="D24" s="4"/>
-      <c r="E24" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F24" s="4"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F24" s="5"/>
     </row>
     <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="4"/>
-      <c r="B25" s="5" t="s">
+      <c r="A25" s="5"/>
+      <c r="B25" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="9">
+      <c r="C25" s="14">
         <v>250000</v>
       </c>
-      <c r="D25" s="4"/>
-      <c r="E25" s="5" t="s">
+      <c r="D25" s="5"/>
+      <c r="E25" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="4"/>
+      <c r="F25" s="5"/>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
+      <c r="A26" s="5"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="4"/>
-      <c r="B27" s="5" t="s">
+      <c r="A27" s="5"/>
+      <c r="B27" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="14">
         <f>SUM(C4:C25)</f>
         <v>9825000</v>
       </c>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BF5CBD5-178D-0A40-B587-3EA86FFC7A75}">
+  <dimension ref="B1:O46"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="0.5" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="0.5" customWidth="1"/>
+    <col min="9" max="9" width="15.5" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="0.5" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="13" max="13" width="0.5" customWidth="1"/>
+    <col min="14" max="14" width="15.5" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="6.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B1" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+    </row>
+    <row r="2" spans="2:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
+      <c r="N2" s="20"/>
+      <c r="O2" s="20"/>
+    </row>
+    <row r="3" spans="2:15" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="21"/>
+    </row>
+    <row r="4" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="27" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="27"/>
+      <c r="G4" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="I4" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="27"/>
+      <c r="L4" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="N4" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="O4" s="27"/>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="C5" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" s="48" t="s">
+        <v>60</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="L5" s="48" t="s">
+        <v>60</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="49" t="s">
+        <v>80</v>
+      </c>
+      <c r="I6" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="J6" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="L6" s="49" t="s">
+        <v>81</v>
+      </c>
+      <c r="N6" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="O6" s="18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B7" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="30"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="31"/>
+      <c r="J7" s="30"/>
+      <c r="K7" s="32"/>
+      <c r="L7" s="47"/>
+      <c r="M7" s="32"/>
+      <c r="N7" s="30"/>
+      <c r="O7" s="33"/>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B8" s="38" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="16">
+        <f>'Sidekick Cap Table'!G4</f>
+        <v>3600000</v>
+      </c>
+      <c r="D8" s="25"/>
+      <c r="E8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="I8" s="25"/>
+      <c r="J8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="N8" s="15">
+        <f>C8+E8+G8+J8+L8</f>
+        <v>3600000</v>
+      </c>
+      <c r="O8" s="42">
+        <f ca="1">N8/$N$31</f>
+        <v>0.19407534339071297</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B9" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="16">
+        <f>'Sidekick Cap Table'!G5</f>
+        <v>3600000</v>
+      </c>
+      <c r="D9" s="25"/>
+      <c r="E9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="I9" s="25"/>
+      <c r="J9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="N9" s="15">
+        <f>C9+E9+G9+J9+L9</f>
+        <v>3600000</v>
+      </c>
+      <c r="O9" s="42">
+        <f ca="1">N9/$N$31</f>
+        <v>0.19407534339071297</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B10" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="16">
+        <f>'Sidekick Cap Table'!G7</f>
+        <v>592500</v>
+      </c>
+      <c r="D10" s="25"/>
+      <c r="E10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="N10" s="15">
+        <f>C10+E10+G10+J10+L10</f>
+        <v>592500</v>
+      </c>
+      <c r="O10" s="42">
+        <f ca="1">N10/$N$31</f>
+        <v>3.1941566933054839E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B11" s="38" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="16">
+        <f>'Sidekick Cap Table'!G8</f>
+        <v>592500</v>
+      </c>
+      <c r="D11" s="25"/>
+      <c r="E11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="15"/>
+      <c r="L11" s="15"/>
+      <c r="N11" s="15">
+        <f>C11+E11+G11+J11+L11</f>
+        <v>592500</v>
+      </c>
+      <c r="O11" s="42">
+        <f ca="1">N11/$N$31</f>
+        <v>3.1941566933054839E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B12" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="16">
+        <f>'Sidekick Cap Table'!G14</f>
+        <v>285000</v>
+      </c>
+      <c r="D12" s="25"/>
+      <c r="E12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="I12" s="25"/>
+      <c r="J12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="N12" s="15">
+        <f>C12+E12+G12+J12+L12</f>
+        <v>285000</v>
+      </c>
+      <c r="O12" s="42">
+        <f ca="1">N12/$N$31</f>
+        <v>1.5364298018431442E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B13" s="38" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="16">
+        <f>'Sidekick Cap Table'!G16</f>
+        <v>285000</v>
+      </c>
+      <c r="D13" s="25"/>
+      <c r="E13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="I13" s="25"/>
+      <c r="J13" s="15"/>
+      <c r="L13" s="15"/>
+      <c r="N13" s="15">
+        <f>C13+E13+G13+J13+L13</f>
+        <v>285000</v>
+      </c>
+      <c r="O13" s="42">
+        <f ca="1">N13/$N$31</f>
+        <v>1.5364298018431442E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B14" s="38" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="16">
+        <f>'Sidekick Cap Table'!G6</f>
+        <v>222187</v>
+      </c>
+      <c r="D14" s="25"/>
+      <c r="E14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="15"/>
+      <c r="L14" s="15"/>
+      <c r="N14" s="15">
+        <f>C14+E14+G14+J14+L14</f>
+        <v>222187</v>
+      </c>
+      <c r="O14" s="42">
+        <f ca="1">N14/$N$31</f>
+        <v>1.1978060644986762E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B15" s="38" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="16">
+        <f>'Sidekick Cap Table'!G9</f>
+        <v>112400</v>
+      </c>
+      <c r="D15" s="25"/>
+      <c r="E15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="15"/>
+      <c r="L15" s="15"/>
+      <c r="N15" s="15">
+        <f>C15+E15+G15+J15+L15</f>
+        <v>112400</v>
+      </c>
+      <c r="O15" s="42">
+        <f ca="1">N15/$N$31</f>
+        <v>6.0594634991989272E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B16" s="38" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="16">
+        <f>'Sidekick Cap Table'!G10+'Sidekick Cap Table'!G11+'Sidekick Cap Table'!G12+'Sidekick Cap Table'!G13+'Sidekick Cap Table'!G15+'Sidekick Cap Table'!G17+'Sidekick Cap Table'!G18+'Sidekick Cap Table'!G19+'Sidekick Cap Table'!G20</f>
+        <v>385571</v>
+      </c>
+      <c r="D16" s="25"/>
+      <c r="E16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="15"/>
+      <c r="L16" s="15"/>
+      <c r="N16" s="15">
+        <f>C16+E16+G16+J16+L16</f>
+        <v>385571</v>
+      </c>
+      <c r="O16" s="42">
+        <f ca="1">N16/$N$31</f>
+        <v>2.0786062285139052E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B17" s="39"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="15"/>
+      <c r="L17" s="15"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="42"/>
+    </row>
+    <row r="18" spans="2:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="38" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="15"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="15"/>
+      <c r="G18" s="16">
+        <f>'Sidekick Cap Table'!G21</f>
+        <v>65105</v>
+      </c>
+      <c r="I18" s="25"/>
+      <c r="J18" s="15"/>
+      <c r="L18" s="15">
+        <f ca="1">IFERROR(ROUND($C$46*N31,0)-G18,0)</f>
+        <v>1789845</v>
+      </c>
+      <c r="N18" s="15">
+        <f ca="1">C18+E18+G18+J18+L18</f>
+        <v>1854950</v>
+      </c>
+      <c r="O18" s="42">
+        <f ca="1">N18/$N$31</f>
+        <v>0.10000001617294528</v>
+      </c>
+    </row>
+    <row r="19" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B19" s="38" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="28">
+        <f>SUM(C8:C18)</f>
+        <v>9675158</v>
+      </c>
+      <c r="D19" s="25">
+        <f>SUM(D8:D18)</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="15">
+        <f>SUM(E8:E18)</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="28">
+        <f>SUM(G8:G18)</f>
+        <v>65105</v>
+      </c>
+      <c r="I19" s="25">
+        <f>SUM(I8:I18)</f>
+        <v>0</v>
+      </c>
+      <c r="J19" s="15">
+        <f>SUM(J8:J18)</f>
+        <v>0</v>
+      </c>
+      <c r="L19" s="28">
+        <f ca="1">SUM(L8:L18)</f>
+        <v>1789845</v>
+      </c>
+      <c r="N19" s="28">
+        <f ca="1">SUM(N8:N18)</f>
+        <v>11530108</v>
+      </c>
+      <c r="O19" s="43">
+        <f ca="1">N19/$N$31</f>
+        <v>0.62158601928666857</v>
+      </c>
+    </row>
+    <row r="20" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B20" s="40" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="15"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="15"/>
+      <c r="L20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="42"/>
+    </row>
+    <row r="21" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B21" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="15"/>
+      <c r="D21" s="50">
+        <f>'SAFE Investments'!C6+'SAFE Investments'!C7+'SAFE Investments'!C8+'SAFE Investments'!C15+'SAFE Investments'!C16+'SAFE Investments'!C17+'SAFE Investments'!C21+'SAFE Investments'!C24</f>
+        <v>8000000</v>
+      </c>
+      <c r="E21" s="15">
+        <f>IFERROR(ROUND(D21/$E$33,0),0)</f>
+        <v>1939567</v>
+      </c>
+      <c r="G21" s="15"/>
+      <c r="I21" s="25">
+        <f>$C$44</f>
+        <v>5000000</v>
+      </c>
+      <c r="J21" s="15">
+        <f ca="1">IFERROR(ROUND(I21/$J$33,0),0)</f>
+        <v>1159340</v>
+      </c>
+      <c r="L21" s="15"/>
+      <c r="N21" s="15">
+        <f ca="1">C21+E21+J21</f>
+        <v>3098907</v>
+      </c>
+      <c r="O21" s="42">
+        <f ca="1">N21/$N$31</f>
+        <v>0.16706151115580115</v>
+      </c>
+    </row>
+    <row r="22" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B22" s="38" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="15"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="I22" s="25">
+        <f>$C$43</f>
+        <v>12000000</v>
+      </c>
+      <c r="J22" s="15">
+        <f ca="1">IFERROR(ROUND(I22/$J$33,0),0)</f>
+        <v>2782415</v>
+      </c>
+      <c r="L22" s="15"/>
+      <c r="N22" s="15">
+        <f ca="1">C22+E22+J22</f>
+        <v>2782415</v>
+      </c>
+      <c r="O22" s="42">
+        <f ca="1">N22/$N$31</f>
+        <v>0.14999948516124184</v>
+      </c>
+    </row>
+    <row r="23" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B23" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="C23" s="15"/>
+      <c r="D23" s="50">
+        <f>'SAFE Investments'!C9</f>
+        <v>250000</v>
+      </c>
+      <c r="E23" s="15">
+        <f>IFERROR(ROUND(D23/$E$33,0),0)</f>
+        <v>60611</v>
+      </c>
+      <c r="G23" s="15"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="15"/>
+      <c r="L23" s="15"/>
+      <c r="N23" s="15">
+        <f>C23+E23+J23</f>
+        <v>60611</v>
+      </c>
+      <c r="O23" s="42">
+        <f ca="1">N23/$N$31</f>
+        <v>3.2675279550706954E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B24" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" s="15"/>
+      <c r="D24" s="50">
+        <f>'SAFE Investments'!C11</f>
+        <v>300000</v>
+      </c>
+      <c r="E24" s="15">
+        <f>IFERROR(ROUND(D24/$E$33,0),0)</f>
+        <v>72734</v>
+      </c>
+      <c r="G24" s="15"/>
+      <c r="I24" s="25"/>
+      <c r="J24" s="15"/>
+      <c r="L24" s="15"/>
+      <c r="N24" s="15">
+        <f>C24+E24+J24</f>
+        <v>72734</v>
+      </c>
+      <c r="O24" s="42">
+        <f ca="1">N24/$N$31</f>
+        <v>3.9210766739389211E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B25" s="38" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="15"/>
+      <c r="D25" s="50">
+        <f>'SAFE Investments'!C13</f>
+        <v>250000</v>
+      </c>
+      <c r="E25" s="15">
+        <f>IFERROR(ROUND(D25/$E$33,0),0)</f>
+        <v>60611</v>
+      </c>
+      <c r="G25" s="15"/>
+      <c r="I25" s="25"/>
+      <c r="J25" s="15"/>
+      <c r="L25" s="15"/>
+      <c r="N25" s="15">
+        <f>C25+E25+J25</f>
+        <v>60611</v>
+      </c>
+      <c r="O25" s="42">
+        <f ca="1">N25/$N$31</f>
+        <v>3.2675279550706954E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B26" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="15"/>
+      <c r="D26" s="50">
+        <f>'SAFE Investments'!C19</f>
+        <v>212500</v>
+      </c>
+      <c r="E26" s="15">
+        <f>IFERROR(ROUND(D26/$E$33,0),0)</f>
+        <v>51520</v>
+      </c>
+      <c r="G26" s="15"/>
+      <c r="I26" s="25"/>
+      <c r="J26" s="15"/>
+      <c r="L26" s="15"/>
+      <c r="N26" s="15">
+        <f>C26+E26+J26</f>
+        <v>51520</v>
+      </c>
+      <c r="O26" s="42">
+        <f ca="1">N26/$N$31</f>
+        <v>2.7774338031915369E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B27" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="15"/>
+      <c r="D27" s="50">
+        <f>'SAFE Investments'!C25</f>
+        <v>250000</v>
+      </c>
+      <c r="E27" s="15">
+        <f>IFERROR(ROUND(D27/$E$33,0),0)</f>
+        <v>60611</v>
+      </c>
+      <c r="G27" s="15"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="15"/>
+      <c r="L27" s="15"/>
+      <c r="N27" s="15">
+        <f>C27+E27+J27</f>
+        <v>60611</v>
+      </c>
+      <c r="O27" s="42">
+        <f ca="1">N27/$N$31</f>
+        <v>3.2675279550706954E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B28" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" s="15"/>
+      <c r="D28" s="50">
+        <f>'SAFE Investments'!C4+'SAFE Investments'!C5+'SAFE Investments'!C10+'SAFE Investments'!C12+'SAFE Investments'!C14+'SAFE Investments'!C18+'SAFE Investments'!C20+'SAFE Investments'!C22+'SAFE Investments'!C23</f>
+        <v>562500</v>
+      </c>
+      <c r="E28" s="15">
+        <f>IFERROR(ROUND(D28/$E$33,0),0)</f>
+        <v>136376</v>
+      </c>
+      <c r="G28" s="15"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="15"/>
+      <c r="L28" s="15"/>
+      <c r="N28" s="15">
+        <f>C28+E28+J28</f>
+        <v>136376</v>
+      </c>
+      <c r="O28" s="42">
+        <f ca="1">N28/$N$31</f>
+        <v>7.3520052861810754E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B29" s="38" t="s">
+        <v>70</v>
+      </c>
+      <c r="C29" s="15"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="I29" s="25">
+        <f>$C$45</f>
+        <v>3000000</v>
+      </c>
+      <c r="J29" s="15">
+        <f ca="1">IFERROR(ROUND(I29/$J$33,0),0)</f>
+        <v>695604</v>
+      </c>
+      <c r="L29" s="15"/>
+      <c r="N29" s="15">
+        <f ca="1">C29+E29+J29</f>
+        <v>695604</v>
+      </c>
+      <c r="O29" s="42">
+        <f ca="1">N29/$N$31</f>
+        <v>3.7499884767764863E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B30" s="39"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="15"/>
+      <c r="L30" s="15"/>
+      <c r="N30" s="15"/>
+      <c r="O30" s="42"/>
+    </row>
+    <row r="31" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B31" s="38" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="34">
+        <f>C19+SUM(C21:C29)</f>
+        <v>9675158</v>
+      </c>
+      <c r="D31" s="35">
+        <f>SUM(D8:D29)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E31" s="34">
+        <f>SUM(E8:E29)</f>
+        <v>2382030</v>
+      </c>
+      <c r="G31" s="34">
+        <f>G18</f>
+        <v>65105</v>
+      </c>
+      <c r="I31" s="35">
+        <f>SUM(I21:I30)</f>
+        <v>20000000</v>
+      </c>
+      <c r="J31" s="34">
+        <f ca="1">SUM(J21:J30)</f>
+        <v>4637359</v>
+      </c>
+      <c r="L31" s="34">
+        <f ca="1">L18</f>
+        <v>1789845</v>
+      </c>
+      <c r="N31" s="34">
+        <f ca="1">SUM(N21:N30)+N19</f>
+        <v>18549497</v>
+      </c>
+      <c r="O31" s="44">
+        <f ca="1">SUM(O21:O29)+O19</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:15" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="39"/>
+      <c r="O32" s="45"/>
+    </row>
+    <row r="33" spans="2:15" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="38" t="s">
+        <v>72</v>
+      </c>
+      <c r="E33" s="22">
+        <f>($C$42-D31)/'Sidekick Cap Table'!G23</f>
+        <v>4.1246319529565065</v>
+      </c>
+      <c r="J33" s="23">
+        <f ca="1">IFERROR(ROUND(J35/N31,4),0)</f>
+        <v>4.3128000000000002</v>
+      </c>
+      <c r="O33" s="45"/>
+    </row>
+    <row r="34" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B34" s="38" t="s">
+        <v>73</v>
+      </c>
+      <c r="J34" s="24">
+        <f>J35-I31</f>
+        <v>60000000</v>
+      </c>
+      <c r="O34" s="45"/>
+    </row>
+    <row r="35" spans="2:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="41" t="s">
+        <v>74</v>
+      </c>
+      <c r="C35" s="36"/>
+      <c r="D35" s="36"/>
+      <c r="E35" s="36"/>
+      <c r="F35" s="36"/>
+      <c r="G35" s="36"/>
+      <c r="H35" s="36"/>
+      <c r="I35" s="36"/>
+      <c r="J35" s="37">
+        <f>C39+C40</f>
+        <v>80000000</v>
+      </c>
+      <c r="K35" s="36"/>
+      <c r="L35" s="36"/>
+      <c r="M35" s="36"/>
+      <c r="N35" s="36"/>
+      <c r="O35" s="46"/>
+    </row>
+    <row r="37" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B37" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B39" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C39" s="17">
+        <v>60000000</v>
+      </c>
+    </row>
+    <row r="40" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B40" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C40" s="17">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="41" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B41" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" s="1">
+        <f>I31/J35</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="42" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B42" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C42" s="17">
+        <v>50000000</v>
+      </c>
+    </row>
+    <row r="43" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B43" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C43" s="17">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="44" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B44" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C44" s="17">
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="45" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B45" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C45" s="17">
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="46" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B46" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C46" s="8">
+        <v>0.1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Checkpoint: Sidekick Cap Table and SAFE Investments sheets complete
</commit_message>
<xml_diff>
--- a/runs/resume/models/model.xlsx
+++ b/runs/resume/models/model.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{707DD6DB-5717-2D45-8F4C-971C50E33FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{09B9779D-D826-3848-823B-68ADCC5EF376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="__temp__" sheetId="82" r:id="rId1"/>
-    <sheet name="Sidekick Cap Table" sheetId="83" r:id="rId2"/>
-    <sheet name="SAFE Investments" sheetId="84" r:id="rId3"/>
+    <sheet name="__temp__" sheetId="89" r:id="rId1"/>
+    <sheet name="Sidekick Cap Table" sheetId="90" r:id="rId2"/>
+    <sheet name="SAFE Investments" sheetId="91" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -133,6 +133,9 @@
     <t>Amir Bagherzadeh</t>
   </si>
   <si>
+    <t>Transfer from Owl Rock Capital II, LLC (Accomplice)</t>
+  </si>
+  <si>
     <t>Elizabeth A. Donaghey Irrevocable Trust 2016</t>
   </si>
   <si>
@@ -191,9 +194,6 @@
   </si>
   <si>
     <t>Mark Lotke</t>
-  </si>
-  <si>
-    <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
   </si>
 </sst>
 </file>
@@ -340,14 +340,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -693,7 +693,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -705,6 +705,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1102,7 +1105,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDE8945D-6B4E-314B-9D0B-93DB3B2B1983}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{264E6C63-5657-C948-958C-E4037E66E6DC}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
@@ -1112,8 +1115,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{829EEB16-14D0-C14F-8C0F-9E7ACFBD646A}">
-  <dimension ref="A1:I23"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30783E96-F939-2244-BC0C-35D6D5C04F42}">
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5" customWidth="1"/>
@@ -1125,9 +1128,10 @@
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="3.33203125" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1137,8 +1141,9 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J1" s="1"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1150,8 +1155,9 @@
         <v>1</v>
       </c>
       <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="2" t="s">
         <v>2</v>
@@ -1175,8 +1181,9 @@
         <v>7</v>
       </c>
       <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>8</v>
@@ -1195,9 +1202,10 @@
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I4" s="4"/>
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>9</v>
@@ -1216,9 +1224,10 @@
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I5" s="4"/>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
         <v>10</v>
@@ -1237,9 +1246,10 @@
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I6" s="4"/>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
         <v>11</v>
@@ -1258,9 +1268,10 @@
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I7" s="4"/>
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
         <v>12</v>
@@ -1279,9 +1290,10 @@
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I8" s="4"/>
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
         <v>13</v>
@@ -1302,9 +1314,10 @@
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I9" s="4"/>
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
         <v>14</v>
@@ -1323,9 +1336,10 @@
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I10" s="4"/>
+      <c r="J10" s="1"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="1" t="s">
         <v>15</v>
@@ -1344,9 +1358,10 @@
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I11" s="4"/>
+      <c r="J11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
         <v>16</v>
@@ -1365,9 +1380,10 @@
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="1"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I12" s="4"/>
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
         <v>17</v>
@@ -1386,9 +1402,10 @@
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I13" s="4"/>
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
       <c r="B14" s="1" t="s">
         <v>18</v>
@@ -1407,9 +1424,10 @@
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I14" s="4"/>
+      <c r="J14" s="1"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
         <v>19</v>
@@ -1428,9 +1446,10 @@
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="1"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I15" s="4"/>
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
         <v>20</v>
@@ -1449,9 +1468,10 @@
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I16" s="4"/>
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="1" t="s">
         <v>21</v>
@@ -1470,9 +1490,10 @@
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I17" s="4"/>
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
         <v>22</v>
@@ -1491,9 +1512,10 @@
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="1"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I18" s="4"/>
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
         <v>23</v>
@@ -1512,9 +1534,10 @@
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="1"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I19" s="4"/>
+      <c r="J19" s="1"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="1" t="s">
         <v>24</v>
@@ -1533,9 +1556,10 @@
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="1"/>
-    </row>
-    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I20" s="4"/>
+      <c r="J20" s="1"/>
+    </row>
+    <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
         <v>25</v>
@@ -1554,20 +1578,22 @@
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="1"/>
-    </row>
-    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I21" s="4"/>
+      <c r="J21" s="1"/>
+    </row>
+    <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-    </row>
-    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G22" s="3"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="1"/>
+    </row>
+    <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="2" t="s">
         <v>0</v>
@@ -1592,8 +1618,12 @@
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
+      <c r="H23" s="3">
+        <f>SUM(H4:H21)</f>
+        <v>0.99999999999999967</v>
+      </c>
+      <c r="I23" s="3"/>
+      <c r="J23" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1601,8 +1631,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C48FF8DF-3B87-E946-A270-300A465EC45E}">
-  <dimension ref="A1:E27"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F79D649-336D-B245-9EE3-22E20CA4CC2C}">
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5" customWidth="1"/>
@@ -1610,317 +1640,345 @@
     <col min="3" max="3" width="12.33203125" customWidth="1"/>
     <col min="4" max="4" width="3.33203125" customWidth="1"/>
     <col min="5" max="5" width="60.1640625" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
+      <c r="C1" s="6"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
+      <c r="C2" s="5"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>25000</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="6">
         <v>25000</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="6">
         <v>137170.75</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="6">
         <v>3846829.25</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="6">
         <v>16566</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="5">
+        <v>33</v>
+      </c>
+      <c r="C9" s="6">
         <v>250000</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="5">
+        <v>34</v>
+      </c>
+      <c r="C10" s="6">
         <v>100000</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="5">
+        <v>35</v>
+      </c>
+      <c r="C11" s="6">
         <v>300000</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" s="5">
+        <v>36</v>
+      </c>
+      <c r="C12" s="6">
         <v>37500</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="5">
+        <v>38</v>
+      </c>
+      <c r="C13" s="6">
         <v>250000</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
       <c r="B14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="5">
+        <v>39</v>
+      </c>
+      <c r="C14" s="6">
         <v>100000</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-    </row>
-    <row r="15" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="5">
+        <v>40</v>
+      </c>
+      <c r="C15" s="6">
         <v>41164</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+      <c r="F15" s="1"/>
+    </row>
+    <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="5">
+        <v>41</v>
+      </c>
+      <c r="C16" s="6">
         <v>2328778</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" s="5">
+        <v>42</v>
+      </c>
+      <c r="C17" s="6">
         <v>1506000</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+      <c r="F17" s="1"/>
+    </row>
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="5">
+        <v>44</v>
+      </c>
+      <c r="C18" s="6">
         <v>50000</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
-    </row>
-    <row r="19" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F18" s="1"/>
+    </row>
+    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="5">
+        <v>45</v>
+      </c>
+      <c r="C19" s="6">
         <v>212500</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="5">
+        <v>46</v>
+      </c>
+      <c r="C20" s="6">
         <v>25000</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C21" s="5">
+        <v>47</v>
+      </c>
+      <c r="C21" s="6">
         <v>61746</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="5">
+        <v>48</v>
+      </c>
+      <c r="C22" s="6">
         <v>100000</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-    </row>
-    <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C23" s="5">
+        <v>49</v>
+      </c>
+      <c r="C23" s="6">
         <v>100000</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-    </row>
-    <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" s="5">
+        <v>50</v>
+      </c>
+      <c r="C24" s="6">
         <v>61746</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+      <c r="F24" s="1"/>
+    </row>
+    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="5">
+        <v>51</v>
+      </c>
+      <c r="C25" s="6">
         <v>250000</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
+      <c r="C26" s="6"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
-    </row>
-    <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="5">
+      <c r="C27" s="6">
         <f>SUM(C4:C25)</f>
         <v>9825000</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Checkpoint: Sidekick Cap Table and SAFE Investments sheets built
</commit_message>
<xml_diff>
--- a/runs/resume/models/model.xlsx
+++ b/runs/resume/models/model.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{730479F6-35B6-9C40-9122-36EC48E220AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C37D7F27-F383-4042-9320-B31C866CE91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet5" sheetId="99" r:id="rId1"/>
-    <sheet name="Sidekick Cap Table" sheetId="100" r:id="rId2"/>
-    <sheet name="SAFE Investments" sheetId="101" r:id="rId3"/>
+    <sheet name="__temp__" sheetId="103" r:id="rId1"/>
+    <sheet name="Sidekick Cap Table" sheetId="107" r:id="rId2"/>
+    <sheet name="SAFE Investments" sheetId="108" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -203,7 +203,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -353,6 +353,13 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -699,7 +706,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -719,10 +726,13 @@
     <xf numFmtId="10" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1117,17 +1127,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21971E0D-EB27-BD40-8182-AFF2F1722D11}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D555A474-5AC6-5048-8F91-0C2401531367}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B934312C-C418-6E4D-B6BA-168ACA963A1D}">
-  <dimension ref="A1:J23"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94114CF6-BCC7-AB4D-951F-13187FA7A0F6}">
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5" customWidth="1"/>
@@ -1142,7 +1153,7 @@
     <col min="10" max="10" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1153,8 +1164,13 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1167,8 +1183,13 @@
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="4" t="s">
         <v>2</v>
@@ -1193,8 +1214,13 @@
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="3" t="s">
         <v>8</v>
@@ -1215,8 +1241,13 @@
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="3" t="s">
         <v>9</v>
@@ -1237,8 +1268,13 @@
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="3" t="s">
         <v>10</v>
@@ -1259,8 +1295,13 @@
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="3" t="s">
         <v>11</v>
@@ -1281,8 +1322,13 @@
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="3" t="s">
         <v>12</v>
@@ -1303,8 +1349,13 @@
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="3" t="s">
         <v>13</v>
@@ -1327,8 +1378,13 @@
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="3" t="s">
         <v>14</v>
@@ -1349,8 +1405,13 @@
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="3" t="s">
         <v>15</v>
@@ -1371,8 +1432,13 @@
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
       <c r="B12" s="3" t="s">
         <v>16</v>
@@ -1393,8 +1459,13 @@
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="3" t="s">
         <v>17</v>
@@ -1415,8 +1486,13 @@
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
       <c r="B14" s="3" t="s">
         <v>18</v>
@@ -1437,8 +1513,13 @@
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="3" t="s">
         <v>19</v>
@@ -1459,8 +1540,13 @@
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="3" t="s">
         <v>20</v>
@@ -1481,8 +1567,13 @@
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="3" t="s">
         <v>21</v>
@@ -1503,8 +1594,13 @@
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="3" t="s">
         <v>22</v>
@@ -1525,8 +1621,13 @@
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="3" t="s">
         <v>23</v>
@@ -1547,8 +1648,13 @@
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="3" t="s">
         <v>24</v>
@@ -1569,8 +1675,13 @@
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
-    </row>
-    <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+    </row>
+    <row r="21" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="3" t="s">
         <v>25</v>
@@ -1591,8 +1702,13 @@
       </c>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
-    </row>
-    <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+    </row>
+    <row r="22" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1600,11 +1716,16 @@
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
       <c r="J22" s="1"/>
-    </row>
-    <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+    </row>
+    <row r="23" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="4" t="s">
         <v>0</v>
@@ -1629,9 +1750,17 @@
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
+      <c r="H23" s="2">
+        <f>SUM(H4:H21)</f>
+        <v>0.99999999999999967</v>
+      </c>
+      <c r="I23" s="1"/>
       <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1639,8 +1768,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E761F8A-3E33-304F-A5DF-2C6DCC25A139}">
-  <dimension ref="A1:F27"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CD2AF51-D88B-FB4D-8BAB-71B43D9CC9D8}">
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5" customWidth="1"/>
@@ -1651,28 +1780,38 @@
     <col min="6" max="6" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="9" t="s">
         <v>26</v>
       </c>
       <c r="D3" s="1"/>
@@ -1680,13 +1819,18 @@
         <v>27</v>
       </c>
       <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="8">
         <v>25000</v>
       </c>
       <c r="D4" s="1"/>
@@ -1694,49 +1838,69 @@
         <v>28</v>
       </c>
       <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="8">
         <v>25000</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="3"/>
       <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="8">
         <v>137170.75</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="3"/>
       <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="8">
         <v>3846829.25</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="3"/>
       <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="8">
         <v>16566</v>
       </c>
       <c r="D8" s="1"/>
@@ -1744,37 +1908,52 @@
         <v>52</v>
       </c>
       <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+    </row>
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="8">
         <v>250000</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="3"/>
       <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+    </row>
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="8">
         <v>100000</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="3"/>
       <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+    </row>
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="8">
         <v>300000</v>
       </c>
       <c r="D11" s="1"/>
@@ -1782,13 +1961,18 @@
         <v>28</v>
       </c>
       <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
       <c r="B12" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="8">
         <v>37500</v>
       </c>
       <c r="D12" s="1"/>
@@ -1796,37 +1980,52 @@
         <v>36</v>
       </c>
       <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+    </row>
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="8">
         <v>250000</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="3"/>
       <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+    </row>
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
       <c r="B14" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="8">
         <v>100000</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="3"/>
       <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+    </row>
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="8">
         <v>41164</v>
       </c>
       <c r="D15" s="1"/>
@@ -1834,13 +2033,18 @@
         <v>52</v>
       </c>
       <c r="F15" s="1"/>
-    </row>
-    <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="8">
         <v>2328778</v>
       </c>
       <c r="D16" s="1"/>
@@ -1848,13 +2052,18 @@
         <v>52</v>
       </c>
       <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+    </row>
+    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="8">
         <v>1506000</v>
       </c>
       <c r="D17" s="1"/>
@@ -1862,25 +2071,35 @@
         <v>42</v>
       </c>
       <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+    </row>
+    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="8">
         <v>50000</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="3"/>
       <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+    </row>
+    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="8">
         <v>212500</v>
       </c>
       <c r="D19" s="1"/>
@@ -1888,25 +2107,35 @@
         <v>36</v>
       </c>
       <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="8">
         <v>25000</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="3"/>
       <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="8">
         <v>61746</v>
       </c>
       <c r="D21" s="1"/>
@@ -1914,37 +2143,52 @@
         <v>52</v>
       </c>
       <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="7">
+      <c r="C22" s="8">
         <v>100000</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="3"/>
       <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="8">
         <v>100000</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="3"/>
       <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+    </row>
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="8">
         <v>61746</v>
       </c>
       <c r="D24" s="1"/>
@@ -1952,13 +2196,18 @@
         <v>52</v>
       </c>
       <c r="F24" s="1"/>
-    </row>
-    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="8">
         <v>250000</v>
       </c>
       <c r="D25" s="1"/>
@@ -1966,16 +2215,26 @@
         <v>51</v>
       </c>
       <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
-    </row>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+    </row>
+    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
       <c r="B27" s="4" t="s">
         <v>0</v>
@@ -1987,6 +2246,11 @@
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>